<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 07/09/2026 09:16
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$N$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$N$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N33"/>
+  <dimension ref="A1:N35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -776,34 +776,34 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>06/2026</t>
+          <t>77/2026</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Transporte de dos mil metros cúbicos (2.000 m³) de ripio arcilloso destinados al mantenimiento y mejoramiento de caminos de la jurisdicción comunal de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>ADQUISICION DE CAMIONETAS</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>14 de septiembre de 2026 - Hora: 10:00</t>
+          <t>11-09-2026 08:00</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -824,12 +824,12 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>id-85e6cfd11c8a8889</t>
+          <t>id-dff70529581309e6</t>
         </is>
       </c>
     </row>
@@ -844,14 +844,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -861,17 +861,17 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>014/2026</t>
+          <t>06/2026</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
+          <t>Transporte de dos mil metros cúbicos (2.000 m³) de ripio arcilloso destinados al mantenimiento y mejoramiento de caminos de la jurisdicción comunal de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ) - SI ES DECRETADO INHABIL, AL DIA SIGUIENTE HABIL, A LA MISMA HORA Y LUGA</t>
+          <t>14 de septiembre de 2026 - Hora: 10:00</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -879,11 +879,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
-        </is>
-      </c>
+      <c r="J6" s="4" t="inlineStr"/>
       <c r="K6" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -901,7 +897,7 @@
       </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>id-9e58cc9ec0b69356</t>
+          <t>id-85e6cfd11c8a8889</t>
         </is>
       </c>
     </row>
@@ -916,34 +912,34 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>27/2026</t>
+          <t>76/2026</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
+          <t>ADQUICION DE CAMIONES COMPACTADORES DE CARGA TRASERA RSU</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>16 de septiembre de 2026 - Hora: 10:00</t>
+          <t>14-09-2026 08:00</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -964,12 +960,12 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>id-608017f47f903d65</t>
+          <t>id-ccdfae2a7ede4696</t>
         </is>
       </c>
     </row>
@@ -984,14 +980,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SEGUÍ</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1001,25 +997,29 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>014/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”. Apertura de Sobres 17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y entrega en Área de Suministro del Municipio, y también se podrá descargar en el Sitio Oficial Digital Municipal https://www.segui.gob.ar . Edgardo Muller, Presidente Municipal. ID:52321 - F.C. 04-00075716 3 v./03/09/2026</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y </t>
+          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ) - SI ES DECRETADO INHABIL, AL DIA SIGUIENTE HABIL, A LA MISMA HORA Y LUGA</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="J8" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
+        </is>
+      </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>id-90c3d1f38f49418a</t>
+          <t>id-9e58cc9ec0b69356</t>
         </is>
       </c>
     </row>
@@ -1059,7 +1059,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
+          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1069,17 +1069,17 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>015/2026</t>
+          <t>27/2026</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
+          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ) - SI ES DECRETADO INHABIL, AL DIA SIGUIENTE HABIL, A LA MISMA HORA Y LUGA</t>
+          <t>16 de septiembre de 2026 - Hora: 10:00</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -1087,11 +1087,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>$ 90.000,00.- (PESOS NOVENTA MIL CON 00/100)</t>
-        </is>
-      </c>
+      <c r="J9" s="4" t="inlineStr"/>
       <c r="K9" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1109,7 +1105,7 @@
       </c>
       <c r="N9" s="4" t="inlineStr">
         <is>
-          <t>id-74dfdad7e5f9d048</t>
+          <t>id-608017f47f903d65</t>
         </is>
       </c>
     </row>
@@ -1124,14 +1120,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE COLON</t>
+          <t>MUNICIPALIDAD DE SEGUÍ</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1139,27 +1135,27 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr"/>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>08-2026</t>
+        </is>
+      </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
+          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”. Apertura de Sobres 17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y entrega en Área de Suministro del Municipio, y también se podrá descargar en el Sitio Oficial Digital Municipal https://www.segui.gob.ar . Edgardo Muller, Presidente Municipal. ID:52321 - F.C. 04-00075716 3 v./03/09/2026</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>24 de SEPTIEMBRE de 2026</t>
+          <t xml:space="preserve">17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y </t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="inlineStr">
-        <is>
-          <t>Sin Cargo</t>
-        </is>
-      </c>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr"/>
       <c r="K10" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1177,7 +1173,7 @@
       </c>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>id-bc610b64999d147d</t>
+          <t>id-90c3d1f38f49418a</t>
         </is>
       </c>
     </row>
@@ -1192,14 +1188,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MUNICIPIO — PRIMER LLAMADO A:</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1209,17 +1205,17 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>015/2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>LUGAR DE APERTURA DE OFERTAS: – Oficina de Compras, Edificio Municipal, calle Juan D. Perón 232</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>DE OFERTA: 07/09/2026 - 10 HS</t>
+          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ) - SI ES DECRETADO INHABIL, AL DIA SIGUIENTE HABIL, A LA MISMA HORA Y LUGA</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -1229,7 +1225,7 @@
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>$ 90.000,00.- (PESOS NOVENTA MIL CON 00/100)</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr">
@@ -1249,7 +1245,7 @@
       </c>
       <c r="N11" s="4" t="inlineStr">
         <is>
-          <t>id-56a815662b393a4b</t>
+          <t>id-74dfdad7e5f9d048</t>
         </is>
       </c>
     </row>
@@ -1264,14 +1260,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>NOGOYA — COMUNA DISTRITO SAUCE -- NOGOYA</t>
+          <t>MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1279,19 +1275,15 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>1/26</t>
-        </is>
-      </c>
+      <c r="F12" s="4" t="inlineStr"/>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Convocar para la adquisi ción de un Tractor agrícola 0 km, con las siguientes características técnicas: potencia de motor de 130 a 150 HP; doble Tracción, 6 (seis) cilindros; y demás especificación que se encuentran en el pliego de Especificaciones Técnicas</t>
+          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>DE PROPUESTAS: Día Viernes 11 de Septiembre de 2026- a las 10:00 horas en la Sede Comunal de Comuna Distrito Sauce</t>
+          <t>24 de SEPTIEMBRE de 2026</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -1301,7 +1293,7 @@
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">sin costo. Solicitar en la Sede Comunal de Distrito Sauce Nogoya o al </t>
+          <t>Sin Cargo</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
@@ -1321,7 +1313,7 @@
       </c>
       <c r="N12" s="4" t="inlineStr">
         <is>
-          <t>id-328f5a2f67c14702</t>
+          <t>id-bc610b64999d147d</t>
         </is>
       </c>
     </row>
@@ -1343,7 +1335,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
+          <t>MUNICIPIO — PRIMER LLAMADO A:</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1353,17 +1345,17 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>06/26</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
+          <t>LUGAR DE APERTURA DE OFERTAS: – Oficina de Compras, Edificio Municipal, calle Juan D. Perón 232</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
+          <t>DE OFERTA: 07/09/2026 - 10 HS</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -1373,7 +1365,7 @@
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="K13" s="6" t="inlineStr">
@@ -1393,7 +1385,7 @@
       </c>
       <c r="N13" s="4" t="inlineStr">
         <is>
-          <t>id-9dbdaa6090d92bd4</t>
+          <t>id-56a815662b393a4b</t>
         </is>
       </c>
     </row>
@@ -1408,14 +1400,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>NOGOYA — COMUNA DISTRITO SAUCE -- NOGOYA</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1425,17 +1417,17 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>1/26</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
+          <t>Convocar para la adquisi ción de un Tractor agrícola 0 km, con las siguientes características técnicas: potencia de motor de 130 a 150 HP; doble Tracción, 6 (seis) cilindros; y demás especificación que se encuentran en el pliego de Especificaciones Técnicas</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
+          <t>DE PROPUESTAS: Día Viernes 11 de Septiembre de 2026- a las 10:00 horas en la Sede Comunal de Comuna Distrito Sauce</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -1443,21 +1435,29 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr"/>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sin costo. Solicitar en la Sede Comunal de Distrito Sauce Nogoya o al </t>
+        </is>
+      </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr"/>
+      <c r="L14" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="N14" s="4" t="inlineStr">
         <is>
-          <t>id-952aef4c115d8f12</t>
+          <t>id-328f5a2f67c14702</t>
         </is>
       </c>
     </row>
@@ -1479,7 +1479,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1489,17 +1489,17 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>06/26</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
+          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
+          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -1507,21 +1507,29 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr"/>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
+        </is>
+      </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr"/>
+      <c r="L15" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="N15" s="4" t="inlineStr">
         <is>
-          <t>id-885d4847519dfd48</t>
+          <t>id-9dbdaa6090d92bd4</t>
         </is>
       </c>
     </row>
@@ -1531,19 +1539,19 @@
           <t>07/09/2026</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE ORO VERDE</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1551,15 +1559,19 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>08/2026</t>
+        </is>
+      </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>El procedimiento licitatorio regido por el presente pliego tiene por objeto la Licitación Pública N° 03/2026 para la venta de los siguientes bienes municipales: a) MINI RETRO DE TIRO: Marca RICHIGER, Serie A, N° 101. Modelo N° 186. Motor N° 991023899, C. V 7, 50, Modelo 7, 50 DB, RPM 1.500 b) COLECTIVO: Mercedes Benz, dominio UKZ353, modelo 1977 según lo que s e detalla en el Pliego de Bases y Condiciones que forma parte de la presente como Anexo I</t>
+          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>La apertura de sobres se realizará el día 14 de septiembre del 2026 a las 10:00 horas, en la sede municipal</t>
+          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -1567,29 +1579,21 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr">
-        <is>
-          <t>El pliego será gratuito. El mismo se encontrará para su consulta y ent</t>
-        </is>
-      </c>
+      <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="L16" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
+      <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="N16" s="4" t="inlineStr">
         <is>
-          <t>id-ddc4dfb118d357f7</t>
+          <t>id-952aef4c115d8f12</t>
         </is>
       </c>
     </row>
@@ -1599,19 +1603,19 @@
           <t>07/09/2026</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1621,17 +1625,17 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1648,12 +1652,12 @@
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="N17" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-885d4847519dfd48</t>
         </is>
       </c>
     </row>
@@ -1668,14 +1672,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>MUNICIPIO DE ORO VERDE</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1683,19 +1687,15 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>02/2025</t>
-        </is>
-      </c>
+      <c r="F18" s="4" t="inlineStr"/>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>El procedimiento licitatorio regido por el presente pliego tiene por objeto la Licitación Pública N° 03/2026 para la venta de los siguientes bienes municipales: a) MINI RETRO DE TIRO: Marca RICHIGER, Serie A, N° 101. Modelo N° 186. Motor N° 991023899, C. V 7, 50, Modelo 7, 50 DB, RPM 1.500 b) COLECTIVO: Mercedes Benz, dominio UKZ353, modelo 1977 según lo que s e detalla en el Pliego de Bases y Condiciones que forma parte de la presente como Anexo I</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>La apertura de sobres se realizará el día 14 de septiembre del 2026 a las 10:00 horas, en la sede municipal</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1703,21 +1703,29 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr"/>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>El pliego será gratuito. El mismo se encontrará para su consulta y ent</t>
+        </is>
+      </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr"/>
+      <c r="L18" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-ddc4dfb118d357f7</t>
         </is>
       </c>
     </row>
@@ -1749,17 +1757,17 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
@@ -1781,7 +1789,7 @@
       </c>
       <c r="N19" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -1813,17 +1821,17 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
@@ -1845,7 +1853,7 @@
       </c>
       <c r="N20" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
@@ -1875,15 +1883,19 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr"/>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1905,7 +1917,7 @@
       </c>
       <c r="N21" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
@@ -1937,17 +1949,17 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
@@ -1969,7 +1981,7 @@
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -1999,19 +2011,15 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>06/2025</t>
-        </is>
-      </c>
+      <c r="F23" s="4" t="inlineStr"/>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
@@ -2033,7 +2041,7 @@
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -2065,17 +2073,17 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
@@ -2097,7 +2105,7 @@
       </c>
       <c r="N24" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -2129,17 +2137,17 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
@@ -2161,7 +2169,7 @@
       </c>
       <c r="N25" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -2193,17 +2201,17 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>04/2025</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
@@ -2225,7 +2233,7 @@
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
@@ -2240,14 +2248,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2257,17 +2265,17 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
@@ -2275,29 +2283,21 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J27" s="4" t="inlineStr">
-        <is>
-          <t>s in cargo Consultas: comprascomuna6to@hotmail.com Celular: 3444- 4493</t>
-        </is>
-      </c>
+      <c r="J27" s="4" t="inlineStr"/>
       <c r="K27" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="L27" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
+      <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="N27" s="4" t="inlineStr">
         <is>
-          <t>id-511256e6329e386a</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
@@ -2319,27 +2319,27 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
@@ -2356,12 +2356,12 @@
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="N28" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
@@ -2376,14 +2376,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2393,17 +2393,17 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>499/26</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA Nº 499/26: EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
@@ -2411,21 +2411,29 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J29" s="4" t="inlineStr"/>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>s in cargo Consultas: comprascomuna6to@hotmail.com Celular: 3444- 4493</t>
+        </is>
+      </c>
       <c r="K29" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr"/>
+      <c r="L29" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="N29" s="4" t="inlineStr">
         <is>
-          <t>id-f53eab44dba8d43f</t>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
@@ -2440,29 +2448,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>235/26</t>
+          <t>01/26</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Licitación Privada N° 235/26: reparación de cenefas en losas pórticos</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
@@ -2484,12 +2492,12 @@
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>id-22f9c51cdaebefb7</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
@@ -2504,9 +2512,9 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2521,12 +2529,12 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>498/26</t>
+          <t>499/26</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA N° 498/26: reparación de un tramo del cerramiento perimetral del Túnel Subfluvial</t>
+          <t>LICITACIÓN PÚBLICA Nº 499/26: EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
@@ -2553,7 +2561,7 @@
       </c>
       <c r="N31" s="4" t="inlineStr">
         <is>
-          <t>id-46d81e3efd2ae483</t>
+          <t>id-f53eab44dba8d43f</t>
         </is>
       </c>
     </row>
@@ -2575,27 +2583,27 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE — Y PUESTA EN VALOR – ESCUE</t>
+          <t>Túnel Subfluvial</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación Privada</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>235/26</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez</t>
+          <t>Licitación Privada N° 235/26: reparación de cenefas en losas pórticos</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN </t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
@@ -2603,29 +2611,21 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J32" s="4" t="inlineStr">
-        <is>
-          <t>Habilitación: Pesos Ciento Veinte Mil con 0/100 - $ 120.000, 00 - Habi</t>
-        </is>
-      </c>
+      <c r="J32" s="4" t="inlineStr"/>
       <c r="K32" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="L32" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
+      <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Túnel Subfluvial</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>id-f8fab7a7b3a06a2d</t>
+          <t>id-22f9c51cdaebefb7</t>
         </is>
       </c>
     </row>
@@ -2647,62 +2647,198 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
+          <t>Túnel Subfluvial</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>498/26</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>LICITACIÓN PÚBLICA N° 498/26: reparación de un tramo del cerramiento perimetral del Túnel Subfluvial</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr"/>
+      <c r="K33" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Túnel Subfluvial</t>
+        </is>
+      </c>
+      <c r="N33" s="4" t="inlineStr">
+        <is>
+          <t>id-46d81e3efd2ae483</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>07/09/2026</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE — Y PUESTA EN VALOR – ESCUE</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>09/2026</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN </t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>Habilitación: Pesos Ciento Veinte Mil con 0/100 - $ 120.000, 00 - Habi</t>
+        </is>
+      </c>
+      <c r="K34" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="L34" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Boletín Oficial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="N34" s="4" t="inlineStr">
+        <is>
+          <t>id-f8fab7a7b3a06a2d</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>07/09/2026</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
           <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE — TERMINACION ESCUELA Nº 54</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="F35" s="4" t="inlineStr">
         <is>
           <t>10/2026</t>
         </is>
       </c>
-      <c r="G33" s="5" t="inlineStr">
+      <c r="G35" s="5" t="inlineStr">
         <is>
           <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez realizado el depósito/transferenci</t>
         </is>
       </c>
-      <c r="H33" s="4" t="inlineStr">
+      <c r="H35" s="4" t="inlineStr">
         <is>
           <t>de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN N</t>
         </is>
       </c>
-      <c r="I33" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J33" s="4" t="inlineStr">
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
         <is>
           <t>Habilitación: Pesos Ochenta Mil con 0/100 - $ 80.000, 00 - Habilitació</t>
         </is>
       </c>
-      <c r="K33" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="L33" s="6" t="inlineStr">
+      <c r="K35" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="L35" s="6" t="inlineStr">
         <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="M35" t="inlineStr">
         <is>
           <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
-      <c r="N33" s="4" t="inlineStr">
+      <c r="N35" s="4" t="inlineStr">
         <is>
           <t>id-d97b43a99f1e1824</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N33"/>
+  <autoFilter ref="A1:N35"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId2"/>
@@ -2729,29 +2865,33 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId52"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 08/09/2026 08:05
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$N$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$N$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -62,12 +62,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N35"/>
+  <dimension ref="A1:N34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -640,34 +640,34 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SAN JOSÉ</t>
+          <t>CONCORDIA — MUNICIPALIDAD DE PUERTO YERUA</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>1/2026</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>selección de proveedor/es para la adquisición de materiales con destino a la realización de cordón cuneta y badenes de la calle Urquiza entre calles Pueyrredón e Independencia</t>
+          <t>Adquisición de una motoniveladora 0 Km</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>07 de septiembre de 2026 a las 09:00 hs</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="N3" s="4" t="inlineStr">
         <is>
-          <t>id-2b7062803859510f</t>
+          <t>id-61b6e4f9568150b0</t>
         </is>
       </c>
     </row>
@@ -715,27 +715,27 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>CONCORDIA — MUNICIPALIDAD DE PUERTO YERUA</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>1/2026</t>
+          <t>77/2026</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de una motoniveladora 0 Km</t>
+          <t>ADQUISICION DE CAMIONETAS</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>11-09-2026 08:00</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
@@ -756,12 +756,12 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>id-61b6e4f9568150b0</t>
+          <t>id-dff70529581309e6</t>
         </is>
       </c>
     </row>
@@ -776,34 +776,34 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>77/2026</t>
+          <t>06/2026</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICION DE CAMIONETAS</t>
+          <t>Transporte de dos mil metros cúbicos (2.000 m³) de ripio arcilloso destinados al mantenimiento y mejoramiento de caminos de la jurisdicción comunal de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>11-09-2026 08:00</t>
+          <t>14 de septiembre de 2026 - Hora: 10:00</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -824,12 +824,12 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>id-dff70529581309e6</t>
+          <t>id-85e6cfd11c8a8889</t>
         </is>
       </c>
     </row>
@@ -844,34 +844,34 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>06/2026</t>
+          <t>76/2026</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Transporte de dos mil metros cúbicos (2.000 m³) de ripio arcilloso destinados al mantenimiento y mejoramiento de caminos de la jurisdicción comunal de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>ADQUICION DE CAMIONES COMPACTADORES DE CARGA TRASERA RSU</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>14 de septiembre de 2026 - Hora: 10:00</t>
+          <t>14-09-2026 08:00</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -892,12 +892,12 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>id-85e6cfd11c8a8889</t>
+          <t>id-ccdfae2a7ede4696</t>
         </is>
       </c>
     </row>
@@ -912,34 +912,34 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>76/2026</t>
+          <t>014/2026</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>ADQUICION DE CAMIONES COMPACTADORES DE CARGA TRASERA RSU</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>14-09-2026 08:00</t>
+          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ) - SI ES DECRETADO INHABIL, AL DIA SIGUIENTE HABIL, A LA MISMA HORA Y LUGA</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -947,7 +947,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr"/>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
+        </is>
+      </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -960,12 +964,12 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>id-ccdfae2a7ede4696</t>
+          <t>id-9e58cc9ec0b69356</t>
         </is>
       </c>
     </row>
@@ -980,14 +984,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
+          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -997,17 +1001,17 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>014/2026</t>
+          <t>27/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
+          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ) - SI ES DECRETADO INHABIL, AL DIA SIGUIENTE HABIL, A LA MISMA HORA Y LUGA</t>
+          <t>16 de septiembre de 2026 - Hora: 10:00</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -1015,11 +1019,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
-        <is>
-          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
-        </is>
-      </c>
+      <c r="J8" s="4" t="inlineStr"/>
       <c r="K8" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>id-9e58cc9ec0b69356</t>
+          <t>id-608017f47f903d65</t>
         </is>
       </c>
     </row>
@@ -1052,14 +1052,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
+          <t>MUNICIPALIDAD DE SEGUÍ</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1069,22 +1069,22 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>27/2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
+          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”. Apertura de Sobres 17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y entrega en Área de Suministro del Municipio, y también se podrá descargar en el Sitio Oficial Digital Municipal https://www.segui.gob.ar . Edgardo Muller, Presidente Municipal. ID:52321 - F.C. 04-00075716 3 v./03/09/2026</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>16 de septiembre de 2026 - Hora: 10:00</t>
+          <t xml:space="preserve">17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y </t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr"/>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="N9" s="4" t="inlineStr">
         <is>
-          <t>id-608017f47f903d65</t>
+          <t>id-90c3d1f38f49418a</t>
         </is>
       </c>
     </row>
@@ -1120,14 +1120,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SEGUÍ</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1137,25 +1137,29 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>015/2026</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”. Apertura de Sobres 17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y entrega en Área de Suministro del Municipio, y también se podrá descargar en el Sitio Oficial Digital Municipal https://www.segui.gob.ar . Edgardo Muller, Presidente Municipal. ID:52321 - F.C. 04-00075716 3 v./03/09/2026</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y </t>
+          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ) - SI ES DECRETADO INHABIL, AL DIA SIGUIENTE HABIL, A LA MISMA HORA Y LUGA</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
+        </is>
+      </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1173,7 +1177,7 @@
       </c>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>id-90c3d1f38f49418a</t>
+          <t>id-74dfdad7e5f9d048</t>
         </is>
       </c>
     </row>
@@ -1188,14 +1192,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1203,19 +1207,15 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>015/2026</t>
-        </is>
-      </c>
+      <c r="F11" s="4" t="inlineStr"/>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
+          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ) - SI ES DECRETADO INHABIL, AL DIA SIGUIENTE HABIL, A LA MISMA HORA Y LUGA</t>
+          <t>24 de SEPTIEMBRE de 2026</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>$ 90.000,00.- (PESOS NOVENTA MIL CON 00/100)</t>
+          <t>Sin Cargo</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr">
@@ -1245,7 +1245,7 @@
       </c>
       <c r="N11" s="4" t="inlineStr">
         <is>
-          <t>id-74dfdad7e5f9d048</t>
+          <t>id-bc610b64999d147d</t>
         </is>
       </c>
     </row>
@@ -1260,14 +1260,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE COLON</t>
+          <t>NOGOYA — COMUNA DISTRITO SAUCE -- NOGOYA</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1275,15 +1275,19 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr"/>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>1/26</t>
+        </is>
+      </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
+          <t>Convocar para la adquisi ción de un Tractor agrícola 0 km, con las siguientes características técnicas: potencia de motor de 130 a 150 HP; doble Tracción, 6 (seis) cilindros; y demás especificación que se encuentran en el pliego de Especificaciones Técnicas</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>24 de SEPTIEMBRE de 2026</t>
+          <t>DE PROPUESTAS: Día Viernes 11 de Septiembre de 2026- a las 10:00 horas en la Sede Comunal de Comuna Distrito Sauce</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -1293,7 +1297,7 @@
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Sin Cargo</t>
+          <t xml:space="preserve">sin costo. Solicitar en la Sede Comunal de Distrito Sauce Nogoya o al </t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
@@ -1313,7 +1317,7 @@
       </c>
       <c r="N12" s="4" t="inlineStr">
         <is>
-          <t>id-bc610b64999d147d</t>
+          <t>id-328f5a2f67c14702</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1339,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MUNICIPIO — PRIMER LLAMADO A:</t>
+          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1345,17 +1349,17 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>06/26</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>LUGAR DE APERTURA DE OFERTAS: – Oficina de Compras, Edificio Municipal, calle Juan D. Perón 232</t>
+          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>DE OFERTA: 07/09/2026 - 10 HS</t>
+          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -1365,7 +1369,7 @@
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
         </is>
       </c>
       <c r="K13" s="6" t="inlineStr">
@@ -1385,7 +1389,7 @@
       </c>
       <c r="N13" s="4" t="inlineStr">
         <is>
-          <t>id-56a815662b393a4b</t>
+          <t>id-9dbdaa6090d92bd4</t>
         </is>
       </c>
     </row>
@@ -1400,14 +1404,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>NOGOYA — COMUNA DISTRITO SAUCE -- NOGOYA</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1417,17 +1421,17 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>1/26</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Convocar para la adquisi ción de un Tractor agrícola 0 km, con las siguientes características técnicas: potencia de motor de 130 a 150 HP; doble Tracción, 6 (seis) cilindros; y demás especificación que se encuentran en el pliego de Especificaciones Técnicas</t>
+          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>DE PROPUESTAS: Día Viernes 11 de Septiembre de 2026- a las 10:00 horas en la Sede Comunal de Comuna Distrito Sauce</t>
+          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -1435,29 +1439,21 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sin costo. Solicitar en la Sede Comunal de Distrito Sauce Nogoya o al </t>
-        </is>
-      </c>
+      <c r="J14" s="4" t="inlineStr"/>
       <c r="K14" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="L14" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
+      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="N14" s="4" t="inlineStr">
         <is>
-          <t>id-328f5a2f67c14702</t>
+          <t>id-952aef4c115d8f12</t>
         </is>
       </c>
     </row>
@@ -1479,7 +1475,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1489,17 +1485,17 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>06/26</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
+          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
+          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -1507,41 +1503,33 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
-        </is>
-      </c>
+      <c r="J15" s="4" t="inlineStr"/>
       <c r="K15" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="L15" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
+      <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="N15" s="4" t="inlineStr">
         <is>
-          <t>id-9dbdaa6090d92bd4</t>
+          <t>id-885d4847519dfd48</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -1551,7 +1539,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1561,17 +1549,17 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
+          <t>DE PROPUESTAS: Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -1579,21 +1567,29 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr"/>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr"/>
+      <c r="L16" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="N16" s="4" t="inlineStr">
         <is>
-          <t>id-952aef4c115d8f12</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
@@ -1603,19 +1599,19 @@
           <t>07/09/2026</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>MUNICIPIO DE ORO VERDE</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1623,19 +1619,15 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>09/2026</t>
-        </is>
-      </c>
+      <c r="F17" s="4" t="inlineStr"/>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
+          <t>El procedimiento licitatorio regido por el presente pliego tiene por objeto la Licitación Pública N° 03/2026 para la venta de los siguientes bienes municipales: a) MINI RETRO DE TIRO: Marca RICHIGER, Serie A, N° 101. Modelo N° 186. Motor N° 991023899, C. V 7, 50, Modelo 7, 50 DB, RPM 1.500 b) COLECTIVO: Mercedes Benz, dominio UKZ353, modelo 1977 según lo que s e detalla en el Pliego de Bases y Condiciones que forma parte de la presente como Anexo I</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
+          <t>La apertura de sobres se realizará el día 14 de septiembre del 2026 a las 10:00 horas, en la sede municipal</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1643,21 +1635,29 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr"/>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>El pliego será gratuito. El mismo se encontrará para su consulta y ent</t>
+        </is>
+      </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr"/>
+      <c r="L17" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="N17" s="4" t="inlineStr">
         <is>
-          <t>id-885d4847519dfd48</t>
+          <t>id-ddc4dfb118d357f7</t>
         </is>
       </c>
     </row>
@@ -1672,14 +1672,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE ORO VERDE</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1687,15 +1687,19 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr"/>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>El procedimiento licitatorio regido por el presente pliego tiene por objeto la Licitación Pública N° 03/2026 para la venta de los siguientes bienes municipales: a) MINI RETRO DE TIRO: Marca RICHIGER, Serie A, N° 101. Modelo N° 186. Motor N° 991023899, C. V 7, 50, Modelo 7, 50 DB, RPM 1.500 b) COLECTIVO: Mercedes Benz, dominio UKZ353, modelo 1977 según lo que s e detalla en el Pliego de Bases y Condiciones que forma parte de la presente como Anexo I</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>La apertura de sobres se realizará el día 14 de septiembre del 2026 a las 10:00 horas, en la sede municipal</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1703,29 +1707,21 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t>El pliego será gratuito. El mismo se encontrará para su consulta y ent</t>
-        </is>
-      </c>
+      <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="L18" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
+      <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>id-ddc4dfb118d357f7</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -1740,7 +1736,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -1757,17 +1753,17 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
@@ -1789,7 +1785,7 @@
       </c>
       <c r="N19" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
@@ -1804,7 +1800,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -1821,17 +1817,17 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
@@ -1853,7 +1849,7 @@
       </c>
       <c r="N20" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
@@ -1868,7 +1864,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -1885,17 +1881,17 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1917,7 +1913,7 @@
       </c>
       <c r="N21" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1928,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -1947,19 +1943,15 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>02/2026</t>
-        </is>
-      </c>
+      <c r="F22" s="4" t="inlineStr"/>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
@@ -1981,7 +1973,7 @@
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -1996,7 +1988,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2011,15 +2003,19 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr"/>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
@@ -2041,7 +2037,7 @@
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -2056,7 +2052,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2073,17 +2069,17 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
@@ -2105,7 +2101,7 @@
       </c>
       <c r="N24" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2116,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2137,17 +2133,17 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
@@ -2169,7 +2165,7 @@
       </c>
       <c r="N25" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2180,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2201,17 +2197,17 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
@@ -2233,7 +2229,7 @@
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2244,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2265,17 +2261,17 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
@@ -2297,7 +2293,7 @@
       </c>
       <c r="N27" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
@@ -2312,14 +2308,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2329,17 +2325,17 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>04/2025</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
@@ -2347,21 +2343,29 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr"/>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>s in cargo Consultas: comprascomuna6to@hotmail.com Celular: 3444- 4493</t>
+        </is>
+      </c>
       <c r="K28" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr"/>
+      <c r="L28" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="N28" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
@@ -2376,34 +2380,34 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>01/26</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
@@ -2411,29 +2415,21 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J29" s="4" t="inlineStr">
-        <is>
-          <t>s in cargo Consultas: comprascomuna6to@hotmail.com Celular: 3444- 4493</t>
-        </is>
-      </c>
+      <c r="J29" s="4" t="inlineStr"/>
       <c r="K29" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="L29" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
+      <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="N29" s="4" t="inlineStr">
         <is>
-          <t>id-511256e6329e386a</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
@@ -2450,27 +2446,27 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>Túnel Subfluvial</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>499/26</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>LICITACIÓN PÚBLICA Nº 499/26: EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
@@ -2492,12 +2488,12 @@
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>Túnel Subfluvial</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-f53eab44dba8d43f</t>
         </is>
       </c>
     </row>
@@ -2512,9 +2508,9 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2524,17 +2520,17 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación Privada</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>499/26</t>
+          <t>235/26</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA Nº 499/26: EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
+          <t>Licitación Privada N° 235/26: reparación de cenefas en losas pórticos</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
@@ -2561,7 +2557,7 @@
       </c>
       <c r="N31" s="4" t="inlineStr">
         <is>
-          <t>id-f53eab44dba8d43f</t>
+          <t>id-22f9c51cdaebefb7</t>
         </is>
       </c>
     </row>
@@ -2588,17 +2584,17 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>235/26</t>
+          <t>498/26</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>Licitación Privada N° 235/26: reparación de cenefas en losas pórticos</t>
+          <t>LICITACIÓN PÚBLICA N° 498/26: reparación de un tramo del cerramiento perimetral del Túnel Subfluvial</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
@@ -2625,7 +2621,7 @@
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>id-22f9c51cdaebefb7</t>
+          <t>id-46d81e3efd2ae483</t>
         </is>
       </c>
     </row>
@@ -2647,7 +2643,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE — Y PUESTA EN VALOR – ESCUE</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2657,17 +2653,17 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>498/26</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA N° 498/26: reparación de un tramo del cerramiento perimetral del Túnel Subfluvial</t>
+          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t xml:space="preserve">de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN </t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
@@ -2675,21 +2671,29 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J33" s="4" t="inlineStr"/>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>Habilitación: Pesos Ciento Veinte Mil con 0/100 - $ 120.000, 00 - Habi</t>
+        </is>
+      </c>
       <c r="K33" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr"/>
+      <c r="L33" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="N33" s="4" t="inlineStr">
         <is>
-          <t>id-46d81e3efd2ae483</t>
+          <t>id-f8fab7a7b3a06a2d</t>
         </is>
       </c>
     </row>
@@ -2711,7 +2715,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE — Y PUESTA EN VALOR – ESCUE</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE — TERMINACION ESCUELA Nº 54</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2721,17 +2725,17 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez</t>
+          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez realizado el depósito/transferenci</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN </t>
+          <t>de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN N</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
@@ -2741,7 +2745,7 @@
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>Habilitación: Pesos Ciento Veinte Mil con 0/100 - $ 120.000, 00 - Habi</t>
+          <t>Habilitación: Pesos Ochenta Mil con 0/100 - $ 80.000, 00 - Habilitació</t>
         </is>
       </c>
       <c r="K34" s="6" t="inlineStr">
@@ -2761,84 +2765,12 @@
       </c>
       <c r="N34" s="4" t="inlineStr">
         <is>
-          <t>id-f8fab7a7b3a06a2d</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>07/09/2026</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE — TERMINACION ESCUELA Nº 54</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>10/2026</t>
-        </is>
-      </c>
-      <c r="G35" s="5" t="inlineStr">
-        <is>
-          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez realizado el depósito/transferenci</t>
-        </is>
-      </c>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t>de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN N</t>
-        </is>
-      </c>
-      <c r="I35" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J35" s="4" t="inlineStr">
-        <is>
-          <t>Habilitación: Pesos Ochenta Mil con 0/100 - $ 80.000, 00 - Habilitació</t>
-        </is>
-      </c>
-      <c r="K35" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="L35" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>Boletín Oficial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="N35" s="4" t="inlineStr">
-        <is>
           <t>id-d97b43a99f1e1824</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N35"/>
+  <autoFilter ref="A1:N34"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId2"/>
@@ -2865,33 +2797,31 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId52"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Columna de apertura como fecha, mejor extracción de venta de pliego y script de planilla con seguimiento
- 'Apertura' ahora es una fecha limpia (dd/mm/aaaa) y el texto largo va en
  'Detalle apertura'. Antes salía todo mezclado y no se podía ordenar.
- parse_fecha acepta '24 DE SEPTIEMBRE DEL AÑO 2026' (formato del Boletín) y
  el boletín busca la fecha en todo el aviso si el campo no la trae:
  las vigentes pasaron de 16 a 19.
- La fecha de venta de pliego se devuelve siempre como dd/mm/aaaa y la ventana
  de búsqueda es más amplia: pasó de 1 a 3 detectadas.
- sheet/Planilla.gs: script de la planilla que baja el CSV y lo vuelca
  preservando las columnas de seguimiento (Presentada/Descartada/Ganada/Perdida,
  precio, posición, notas). Probado: el seguimiento sobrevive a las
  actualizaciones. Arma además una hoja Resumen.
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$N$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N36"/>
+  <dimension ref="A1:O36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -476,13 +476,14 @@
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="70" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="26" customWidth="1" min="13" max="13"/>
-    <col hidden="1" width="1" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
+    <col hidden="1" width="1" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -528,30 +529,35 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>Detalle apertura</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Venta hasta</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Valor pliego</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Pliego PDF</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
@@ -560,7 +566,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -595,35 +601,40 @@
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
           <t>01 de OCTUBRE de 2026 a la hora 10:00 en la Oficina de Compras de la Municipalidad de Villa Elisa, Entre Ríos</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">$ 20.000,00 (Pesos Veinte mil con 00/100) el que se puede adquirir en </t>
         </is>
       </c>
-      <c r="K2" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
       <c r="L2" s="6" t="inlineStr">
         <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M2" s="6" t="inlineStr">
+        <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>id-0132097e777a3442</t>
         </is>
@@ -632,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -672,26 +683,31 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr"/>
-      <c r="K3" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr"/>
       <c r="L3" s="6" t="inlineStr">
         <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="O3" s="4" t="inlineStr">
         <is>
           <t>id-61b6e4f9568150b0</t>
         </is>
@@ -700,7 +716,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -715,60 +731,69 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>NOGOYA — COMUNA DISTRITO SAUCE -- NOGOYA</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>77/2026</t>
+          <t>1/26</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICION DE CAMIONETAS</t>
+          <t>Convocar para la adquisi ción de un Tractor agrícola 0 km, con las siguientes características técnicas: potencia de motor de 130 a 150 HP; doble Tracción, 6 (seis) cilindros; y demás especificación que se encuentran en el pliego de Especificaciones Técnicas</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>11-09-2026 08:00</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr"/>
-      <c r="K4" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
+          <t>Viernes 11 de Septiembre de 2026- a las 10:00 horas en la Sede Comunal de Comuna Distrito Sauce</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sin costo. Solicitar en la Sede Comunal de Distrito Sauce Nogoya o al </t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
         <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M4" s="6" t="inlineStr">
+        <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Municipalidad de Paraná</t>
-        </is>
-      </c>
-      <c r="N4" s="4" t="inlineStr">
-        <is>
-          <t>id-dff70529581309e6</t>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Boletín Oficial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>id-328f5a2f67c14702</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -776,67 +801,72 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>06/2026</t>
+          <t>77/2026</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Transporte de dos mil metros cúbicos (2.000 m³) de ripio arcilloso destinados al mantenimiento y mejoramiento de caminos de la jurisdicción comunal de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>ADQUISICION DE CAMIONETAS</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>14 de septiembre de 2026 - Hora: 10:00</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr"/>
-      <c r="K5" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
+          <t>11-09-2026 08:00</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr"/>
       <c r="L5" s="6" t="inlineStr">
         <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Boletín Oficial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="N5" s="4" t="inlineStr">
-        <is>
-          <t>id-85e6cfd11c8a8889</t>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Municipalidad de Paraná</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>id-dff70529581309e6</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -844,67 +874,72 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>76/2026</t>
+          <t>06/2026</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>ADQUICION DE CAMIONES COMPACTADORES DE CARGA TRASERA RSU</t>
+          <t>Transporte de dos mil metros cúbicos (2.000 m³) de ripio arcilloso destinados al mantenimiento y mejoramiento de caminos de la jurisdicción comunal de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>14-09-2026 08:00</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr"/>
-      <c r="K6" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
+          <t>14 de septiembre de 2026 - Hora: 10:00</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr"/>
       <c r="L6" s="6" t="inlineStr">
         <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M6" s="6" t="inlineStr">
+        <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>Municipalidad de Paraná</t>
-        </is>
-      </c>
-      <c r="N6" s="4" t="inlineStr">
-        <is>
-          <t>id-ccdfae2a7ede4696</t>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Boletín Oficial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>id-85e6cfd11c8a8889</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -912,14 +947,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
+          <t>MUNICIPIO DE ORO VERDE</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -927,56 +962,57 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>014/2026</t>
-        </is>
-      </c>
+      <c r="F7" s="4" t="inlineStr"/>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
+          <t>El procedimiento licitatorio regido por el presente pliego tiene por objeto la Licitación Pública N° 03/2026 para la venta de los siguientes bienes municipales: a) MINI RETRO DE TIRO: Marca RICHIGER, Serie A, N° 101. Modelo N° 186. Motor N° 991023899, C. V 7, 50, Modelo 7, 50 DB, RPM 1.500 b) COLECTIVO: Mercedes Benz, dominio UKZ353, modelo 1977 según lo que s e detalla en el Pliego de Bases y Condiciones que forma parte de la presente como Anexo I</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ) - SI ES DECRETADO INHABIL, AL DIA SIGUIENTE HABIL, A LA MISMA HORA Y LUGA</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>La apertura de sobres se realizará el día 14 de septiembre del 2026 a las 10:00 horas, en la sede municipal</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
-        </is>
-      </c>
-      <c r="K7" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>El pliego será gratuito. El mismo se encontrará para su consulta y ent</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M7" s="6" t="inlineStr">
+        <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
-      <c r="N7" s="4" t="inlineStr">
-        <is>
-          <t>id-9e58cc9ec0b69356</t>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>id-ddc4dfb118d357f7</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -984,67 +1020,72 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>27/2026</t>
+          <t>76/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
+          <t>ADQUICION DE CAMIONES COMPACTADORES DE CARGA TRASERA RSU</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>16 de septiembre de 2026 - Hora: 10:00</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J8" s="4" t="inlineStr"/>
-      <c r="K8" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
+          <t>14-09-2026 08:00</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr"/>
       <c r="L8" s="6" t="inlineStr">
         <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M8" s="6" t="inlineStr">
+        <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>Boletín Oficial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="N8" s="4" t="inlineStr">
-        <is>
-          <t>id-608017f47f903d65</t>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Municipalidad de Paraná</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t>id-ccdfae2a7ede4696</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1052,14 +1093,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SEGUÍ</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1069,50 +1110,59 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>014/2026</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”. Apertura de Sobres 17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y entrega en Área de Suministro del Municipio, y también se podrá descargar en el Sitio Oficial Digital Municipal https://www.segui.gob.ar . Edgardo Muller, Presidente Municipal. ID:52321 - F.C. 04-00075716 3 v./03/09/2026</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y </t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="J9" s="4" t="inlineStr"/>
-      <c r="K9" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
+          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
-      <c r="N9" s="4" t="inlineStr">
-        <is>
-          <t>id-90c3d1f38f49418a</t>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>id-9e58cc9ec0b69356</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1120,14 +1170,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1137,54 +1187,51 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>015/2026</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
+          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ) - SI ES DECRETADO INHABIL, AL DIA SIGUIENTE HABIL, A LA MISMA HORA Y LUGA</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
-        </is>
-      </c>
-      <c r="K10" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr"/>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>Boletín Oficial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="N10" s="4" t="inlineStr">
-        <is>
-          <t>id-74dfdad7e5f9d048</t>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Min. Planeamiento (provincia)</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>id-952aef4c115d8f12</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1199,7 +1246,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1207,45 +1254,50 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr"/>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>27/2026</t>
+        </is>
+      </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
+          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>24 de SEPTIEMBRE de 2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>16 de septiembre de 2026 - Hora: 10:00</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>Sin Cargo</t>
-        </is>
-      </c>
-      <c r="K11" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr"/>
       <c r="L11" s="6" t="inlineStr">
         <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M11" s="6" t="inlineStr">
+        <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
-      <c r="N11" s="4" t="inlineStr">
-        <is>
-          <t>id-bc610b64999d147d</t>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>id-608017f47f903d65</t>
         </is>
       </c>
     </row>
@@ -1267,7 +1319,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ — CONDARCO”</t>
+          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1277,54 +1329,59 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>06/26</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
-      <c r="K12" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M12" s="6" t="inlineStr">
+        <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
-      <c r="N12" s="4" t="inlineStr">
-        <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t>id-9dbdaa6090d92bd4</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1332,14 +1389,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>NOGOYA — COMUNA DISTRITO SAUCE -- NOGOYA</t>
+          <t>MUNICIPALIDAD DE SEGUÍ</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1349,54 +1406,55 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>1/26</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Convocar para la adquisi ción de un Tractor agrícola 0 km, con las siguientes características técnicas: potencia de motor de 130 a 150 HP; doble Tracción, 6 (seis) cilindros; y demás especificación que se encuentran en el pliego de Especificaciones Técnicas</t>
+          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”. Apertura de Sobres 17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y entrega en Área de Suministro del Municipio, y también se podrá descargar en el Sitio Oficial Digital Municipal https://www.segui.gob.ar . Edgardo Muller, Presidente Municipal. ID:52321 - F.C. 04-00075716 3 v./03/09/2026</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>DE PROPUESTAS: Día Viernes 11 de Septiembre de 2026- a las 10:00 horas en la Sede Comunal de Comuna Distrito Sauce</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">sin costo. Solicitar en la Sede Comunal de Distrito Sauce Nogoya o al </t>
-        </is>
-      </c>
-      <c r="K13" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr"/>
       <c r="L13" s="6" t="inlineStr">
         <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M13" s="6" t="inlineStr">
+        <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
-      <c r="N13" s="4" t="inlineStr">
-        <is>
-          <t>id-328f5a2f67c14702</t>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>id-90c3d1f38f49418a</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1404,14 +1462,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1421,54 +1479,59 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>06/26</t>
+          <t>015/2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
-        </is>
-      </c>
-      <c r="K14" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M14" s="6" t="inlineStr">
+        <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
-      <c r="N14" s="4" t="inlineStr">
-        <is>
-          <t>id-9dbdaa6090d92bd4</t>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>id-74dfdad7e5f9d048</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1493,39 +1556,44 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
+          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr"/>
-      <c r="K15" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr">
+          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr"/>
+      <c r="L15" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr">
         <is>
           <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
-      <c r="N15" s="4" t="inlineStr">
-        <is>
-          <t>id-952aef4c115d8f12</t>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t>id-885d4847519dfd48</t>
         </is>
       </c>
     </row>
@@ -1540,14 +1608,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1555,48 +1623,57 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>10/2026</t>
-        </is>
-      </c>
+      <c r="F16" s="4" t="inlineStr"/>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
+          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J16" s="4" t="inlineStr"/>
-      <c r="K16" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>Min. Planeamiento (provincia)</t>
-        </is>
-      </c>
-      <c r="N16" s="4" t="inlineStr">
-        <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>24 de SEPTIEMBRE de 2026</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>Sin Cargo</t>
+        </is>
+      </c>
+      <c r="L16" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M16" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Boletín Oficial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="O16" s="4" t="inlineStr">
+        <is>
+          <t>id-bc610b64999d147d</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1611,7 +1688,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE — TERMINACION ESCUELA Nº 54</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1621,61 +1698,74 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
+          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez realizado el depósito/transferenci</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J17" s="4" t="inlineStr"/>
-      <c r="K17" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>Min. Planeamiento (provincia)</t>
-        </is>
-      </c>
-      <c r="N17" s="4" t="inlineStr">
-        <is>
-          <t>id-885d4847519dfd48</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN N</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>Habilitación: Pesos Ochenta Mil con 0/100 - $ 80.000, 00 - Habilitació</t>
+        </is>
+      </c>
+      <c r="L17" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M17" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Boletín Oficial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="O17" s="4" t="inlineStr">
+        <is>
+          <t>id-d97b43a99f1e1824</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE ORO VERDE</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE — Y PUESTA EN VALOR – ESCUE</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1683,67 +1773,76 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr"/>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>09/2026</t>
+        </is>
+      </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>El procedimiento licitatorio regido por el presente pliego tiene por objeto la Licitación Pública N° 03/2026 para la venta de los siguientes bienes municipales: a) MINI RETRO DE TIRO: Marca RICHIGER, Serie A, N° 101. Modelo N° 186. Motor N° 991023899, C. V 7, 50, Modelo 7, 50 DB, RPM 1.500 b) COLECTIVO: Mercedes Benz, dominio UKZ353, modelo 1977 según lo que s e detalla en el Pliego de Bases y Condiciones que forma parte de la presente como Anexo I</t>
+          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>La apertura de sobres se realizará el día 14 de septiembre del 2026 a las 10:00 horas, en la sede municipal</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>El pliego será gratuito. El mismo se encontrará para su consulta y ent</t>
-        </is>
-      </c>
-      <c r="K18" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>Habilitación: Pesos Ciento Veinte Mil con 0/100 - $ 120.000, 00 - Habi</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
         <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M18" s="6" t="inlineStr">
+        <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
-      <c r="N18" s="4" t="inlineStr">
-        <is>
-          <t>id-ddc4dfb118d357f7</t>
+      <c r="O18" s="4" t="inlineStr">
+        <is>
+          <t>id-f8fab7a7b3a06a2d</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ — CONDARCO”</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1753,61 +1852,74 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J19" s="4" t="inlineStr"/>
-      <c r="K19" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>IAPV — Viviendas</t>
-        </is>
-      </c>
-      <c r="N19" s="4" t="inlineStr">
-        <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
+      <c r="L19" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M19" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Boletín Oficial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1817,46 +1929,51 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J20" s="4" t="inlineStr"/>
-      <c r="K20" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>IAPV — Viviendas</t>
-        </is>
-      </c>
-      <c r="N20" s="4" t="inlineStr">
-        <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr"/>
+      <c r="L20" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Min. Planeamiento (provincia)</t>
+        </is>
+      </c>
+      <c r="O20" s="4" t="inlineStr">
+        <is>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1864,14 +1981,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1881,46 +1998,55 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
-        </is>
-      </c>
+          <t>L LAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr"/>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J21" s="4" t="inlineStr"/>
-      <c r="K21" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>IAPV — Viviendas</t>
-        </is>
-      </c>
-      <c r="N21" s="4" t="inlineStr">
-        <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>Ver boletín</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
+      <c r="L21" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M21" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Boletín Oficial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="O21" s="4" t="inlineStr">
+        <is>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1928,14 +2054,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1945,46 +2071,55 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
-        </is>
-      </c>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr"/>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J22" s="4" t="inlineStr"/>
-      <c r="K22" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>IAPV — Viviendas</t>
-        </is>
-      </c>
-      <c r="N22" s="4" t="inlineStr">
-        <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>Ver boletín</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>s in cargo Consultas: comprascomuna6to@hotmail.com Celular: 3444- 4493</t>
+        </is>
+      </c>
+      <c r="L22" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M22" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Boletín Oficial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="O22" s="4" t="inlineStr">
+        <is>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2007,44 +2142,49 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr"/>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>03/26</t>
+        </is>
+      </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
-        </is>
-      </c>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr"/>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J23" s="4" t="inlineStr"/>
-      <c r="K23" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr">
+          <t>Publicada 21/08/2026 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr"/>
+      <c r="L23" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr">
         <is>
           <t>IAPV — Viviendas</t>
         </is>
       </c>
-      <c r="N23" s="4" t="inlineStr">
-        <is>
-          <t>id-ebeeb6a87e688d85</t>
+      <c r="O23" s="4" t="inlineStr">
+        <is>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2069,46 +2209,47 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
-        </is>
-      </c>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J24" s="4" t="inlineStr"/>
-      <c r="K24" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr">
+          <t>Publicada 09/06/2026 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr"/>
+      <c r="L24" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr">
         <is>
           <t>IAPV — Viviendas</t>
         </is>
       </c>
-      <c r="N24" s="4" t="inlineStr">
-        <is>
-          <t>id-22811eab8859abaf</t>
+      <c r="O24" s="4" t="inlineStr">
+        <is>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2133,46 +2274,47 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
-        </is>
-      </c>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J25" s="4" t="inlineStr"/>
-      <c r="K25" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr">
+          <t>Publicada 05/06/2026 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K25" s="4" t="inlineStr"/>
+      <c r="L25" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr">
         <is>
           <t>IAPV — Viviendas</t>
         </is>
       </c>
-      <c r="N25" s="4" t="inlineStr">
-        <is>
-          <t>id-c019bf4a08989c09</t>
+      <c r="O25" s="4" t="inlineStr">
+        <is>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2197,46 +2339,47 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
-        </is>
-      </c>
+          <t>NOGOYA 19 VIVIENDAS</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J26" s="4" t="inlineStr"/>
-      <c r="K26" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr">
+          <t>Publicada 11/12/2025 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="inlineStr"/>
+      <c r="L26" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr">
         <is>
           <t>IAPV — Viviendas</t>
         </is>
       </c>
-      <c r="N26" s="4" t="inlineStr">
-        <is>
-          <t>id-7c1bf02160a66f67</t>
+      <c r="O26" s="4" t="inlineStr">
+        <is>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2261,46 +2404,47 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
-        </is>
-      </c>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J27" s="4" t="inlineStr"/>
-      <c r="K27" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr">
+          <t>Publicada 18/11/2025 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="inlineStr"/>
+      <c r="L27" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr">
         <is>
           <t>IAPV — Viviendas</t>
         </is>
       </c>
-      <c r="N27" s="4" t="inlineStr">
-        <is>
-          <t>id-2b877612500f72b1</t>
+      <c r="O27" s="4" t="inlineStr">
+        <is>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2323,41 +2467,38 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>04/2025</t>
-        </is>
-      </c>
+      <c r="F28" s="4" t="inlineStr"/>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
-        </is>
-      </c>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J28" s="4" t="inlineStr"/>
-      <c r="K28" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr">
+          <t>Publicada 11/11/2025 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K28" s="4" t="inlineStr"/>
+      <c r="L28" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr">
         <is>
           <t>IAPV — Viviendas</t>
         </is>
       </c>
-      <c r="N28" s="4" t="inlineStr">
-        <is>
-          <t>id-34c85bcdb9b1123f</t>
+      <c r="O28" s="4" t="inlineStr">
+        <is>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -2372,14 +2513,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2389,54 +2530,47 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>L LAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>Ver boletín</t>
-        </is>
-      </c>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
-      <c r="K29" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K29" s="4" t="inlineStr"/>
       <c r="L29" s="6" t="inlineStr">
         <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>Boletín Oficial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="N29" s="4" t="inlineStr">
-        <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O29" s="4" t="inlineStr">
+        <is>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2444,14 +2578,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2461,54 +2595,47 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
-        </is>
-      </c>
-      <c r="H30" s="4" t="inlineStr">
-        <is>
-          <t>Ver boletín</t>
-        </is>
-      </c>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>s in cargo Consultas: comprascomuna6to@hotmail.com Celular: 3444- 4493</t>
-        </is>
-      </c>
-      <c r="K30" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K30" s="4" t="inlineStr"/>
       <c r="L30" s="6" t="inlineStr">
         <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>Boletín Oficial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="N30" s="4" t="inlineStr">
-        <is>
-          <t>id-511256e6329e386a</t>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O30" s="4" t="inlineStr">
+        <is>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2523,56 +2650,57 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
-        </is>
-      </c>
-      <c r="H31" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J31" s="4" t="inlineStr"/>
-      <c r="K31" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="N31" s="4" t="inlineStr">
-        <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K31" s="4" t="inlineStr"/>
+      <c r="L31" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O31" s="4" t="inlineStr">
+        <is>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2580,14 +2708,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2597,46 +2725,47 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>499/26</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA Nº 499/26: EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
-        </is>
-      </c>
-      <c r="H32" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
+          <t>Concurso de Precio N° 02/2025</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J32" s="4" t="inlineStr"/>
-      <c r="K32" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>Túnel Subfluvial</t>
-        </is>
-      </c>
-      <c r="N32" s="4" t="inlineStr">
-        <is>
-          <t>id-f53eab44dba8d43f</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K32" s="4" t="inlineStr"/>
+      <c r="L32" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O32" s="4" t="inlineStr">
+        <is>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2644,63 +2773,64 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C33" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>235/26</t>
+          <t>01/26</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>Licitación Privada N° 235/26: reparación de cenefas en losas pórticos</t>
-        </is>
-      </c>
-      <c r="H33" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J33" s="4" t="inlineStr"/>
-      <c r="K33" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>Túnel Subfluvial</t>
-        </is>
-      </c>
-      <c r="N33" s="4" t="inlineStr">
-        <is>
-          <t>id-22f9c51cdaebefb7</t>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K33" s="4" t="inlineStr"/>
+      <c r="L33" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="O33" s="4" t="inlineStr">
+        <is>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2708,9 +2838,9 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C34" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2725,46 +2855,47 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>498/26</t>
+          <t>499/26</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA N° 498/26: reparación de un tramo del cerramiento perimetral del Túnel Subfluvial</t>
-        </is>
-      </c>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
+          <t>LICITACIÓN PÚBLICA Nº 499/26: EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J34" s="4" t="inlineStr"/>
-      <c r="K34" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr">
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K34" s="4" t="inlineStr"/>
+      <c r="L34" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr">
         <is>
           <t>Túnel Subfluvial</t>
         </is>
       </c>
-      <c r="N34" s="4" t="inlineStr">
-        <is>
-          <t>id-46d81e3efd2ae483</t>
+      <c r="O34" s="4" t="inlineStr">
+        <is>
+          <t>id-f53eab44dba8d43f</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2779,29 +2910,25 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE — Y PUESTA EN VALOR – ESCUE</t>
+          <t>Túnel Subfluvial</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación Privada</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>235/26</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez</t>
-        </is>
-      </c>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN </t>
-        </is>
-      </c>
+          <t>Licitación Privada N° 235/26: reparación de cenefas en losas pórticos</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
           <t>Ver pliego</t>
@@ -2809,34 +2936,31 @@
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>Habilitación: Pesos Ciento Veinte Mil con 0/100 - $ 120.000, 00 - Habi</t>
-        </is>
-      </c>
-      <c r="K35" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="inlineStr"/>
       <c r="L35" s="6" t="inlineStr">
         <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>Boletín Oficial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="N35" s="4" t="inlineStr">
-        <is>
-          <t>id-f8fab7a7b3a06a2d</t>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Túnel Subfluvial</t>
+        </is>
+      </c>
+      <c r="O35" s="4" t="inlineStr">
+        <is>
+          <t>id-22f9c51cdaebefb7</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2851,7 +2975,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE — TERMINACION ESCUELA Nº 54</t>
+          <t>Túnel Subfluvial</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2861,19 +2985,15 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>498/26</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez realizado el depósito/transferenci</t>
-        </is>
-      </c>
-      <c r="H36" s="4" t="inlineStr">
-        <is>
-          <t>de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN N</t>
-        </is>
-      </c>
+          <t>LICITACIÓN PÚBLICA N° 498/26: reparación de un tramo del cerramiento perimetral del Túnel Subfluvial</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
           <t>Ver pliego</t>
@@ -2881,85 +3001,82 @@
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>Habilitación: Pesos Ochenta Mil con 0/100 - $ 80.000, 00 - Habilitació</t>
-        </is>
-      </c>
-      <c r="K36" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K36" s="4" t="inlineStr"/>
       <c r="L36" s="6" t="inlineStr">
         <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>Boletín Oficial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="N36" s="4" t="inlineStr">
-        <is>
-          <t>id-d97b43a99f1e1824</t>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Túnel Subfluvial</t>
+        </is>
+      </c>
+      <c r="O36" s="4" t="inlineStr">
+        <is>
+          <t>id-46d81e3efd2ae483</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N36"/>
+  <autoFilter ref="A1:O36"/>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId53"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Boletín Oficial: 25 días y descarga en paralelo
Mirar 25 días atrás en vez de 10 sube las vigentes de 19 a 24, pero bajar ~16
PDFs de 2 MB en secuencia se pasaba del límite de tiempo y la fuente quedaba
descartada. Ahora se bajan en paralelo (una sesión de requests por hilo, que no
es thread-safe) y el Boletín tiene un límite propio más amplio por ser la fuente
más pesada y la más valiosa.
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -62,12 +62,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O36"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -651,39 +651,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>CONCORDIA — MUNICIPALIDAD DE PUERTO YERUA</t>
+          <t>MUNICIPALIDAD DE CHAJARI — APERTURA: 08 DE SEPTIEMBRE DE 2026 - HORA: 10:00 (DIEZ) - SI ES</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitacion Publica</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>1/2026</t>
+          <t>013/2026</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de una motoniveladora 0 Km</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – hierro y otros – que serán destinados a la construcción de viviendas que se llevarán a cabo en el marco del Plan Construir Futuro 7</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>08 DE SEPTIEMBRE DE 2026 - HORA: 10:00 (DIEZ)</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -691,7 +691,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr"/>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>$ 100.000,00.- (PESOS CIEN MIL CON 00/100) PRESUPUESTO OFICIAL ESTIMAD</t>
+        </is>
+      </c>
       <c r="L3" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -709,7 +713,7 @@
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>id-61b6e4f9568150b0</t>
+          <t>id-2ac90305e5165aad</t>
         </is>
       </c>
     </row>
@@ -724,14 +728,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NOGOYA — COMUNA DISTRITO SAUCE -- NOGOYA</t>
+          <t>FEDERACION — COMUNA DE SAN PEDRO -- DEPARTAMENTO DE FEDERACIÓN</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -741,22 +745,22 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>1/26</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Convocar para la adquisi ción de un Tractor agrícola 0 km, con las siguientes características técnicas: potencia de motor de 130 a 150 HP; doble Tracción, 6 (seis) cilindros; y demás especificación que se encuentran en el pliego de Especificaciones Técnicas</t>
+          <t>“PROVISION RIPIO SELECCIONADO EN ORIGEN Y ENTREGADO SOBRE TRANSPORTE”</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Viernes 11 de Septiembre de 2026- a las 10:00 horas en la Sede Comunal de Comuna Distrito Sauce</t>
+          <t>09 de Septiembre de 2026 - 10:00 hs</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -766,7 +770,7 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">sin costo. Solicitar en la Sede Comunal de Distrito Sauce Nogoya o al </t>
+          <t>Sin costo</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
@@ -786,7 +790,7 @@
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>id-328f5a2f67c14702</t>
+          <t>id-719cc55444d8579b</t>
         </is>
       </c>
     </row>
@@ -808,32 +812,32 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>CONCORDIA — MUNICIPALIDAD DE PUERTO YERUA</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>77/2026</t>
+          <t>1/2026</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICION DE CAMIONETAS</t>
+          <t>Adquisición de una motoniveladora 0 Km</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>11-09-2026 08:00</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -854,12 +858,12 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-dff70529581309e6</t>
+          <t>id-61b6e4f9568150b0</t>
         </is>
       </c>
     </row>
@@ -874,14 +878,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>Áridos</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>ENTE INTERPROVINCIAL TUNEL SUBFLUVIAL RAUL URANGA -- CARLOS S. BEGNIS</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -889,24 +893,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>06/2026</t>
-        </is>
-      </c>
+      <c r="F6" s="4" t="inlineStr"/>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Transporte de dos mil metros cúbicos (2.000 m³) de ripio arcilloso destinados al mantenimiento y mejoramiento de caminos de la jurisdicción comunal de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>14 de septiembre de 2026 - Hora: 10:00</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -914,7 +914,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr"/>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>GRATUITO FECHA DE APERTURA: 10/09/2026</t>
+        </is>
+      </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -932,7 +936,7 @@
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-85e6cfd11c8a8889</t>
+          <t>id-439ddd7aaa7f7b3e</t>
         </is>
       </c>
     </row>
@@ -954,7 +958,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE ORO VERDE</t>
+          <t>NOGOYA — COMUNA DISTRITO SAUCE -- NOGOYA</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -962,20 +966,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr"/>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>1/26</t>
+        </is>
+      </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>El procedimiento licitatorio regido por el presente pliego tiene por objeto la Licitación Pública N° 03/2026 para la venta de los siguientes bienes municipales: a) MINI RETRO DE TIRO: Marca RICHIGER, Serie A, N° 101. Modelo N° 186. Motor N° 991023899, C. V 7, 50, Modelo 7, 50 DB, RPM 1.500 b) COLECTIVO: Mercedes Benz, dominio UKZ353, modelo 1977 según lo que s e detalla en el Pliego de Bases y Condiciones que forma parte de la presente como Anexo I</t>
+          <t>Convocar para la adquisi ción de un Tractor agrícola 0 km, con las siguientes características técnicas: potencia de motor de 130 a 150 HP; doble Tracción, 6 (seis) cilindros; y demás especificación que se encuentran en el pliego de Especificaciones Técnicas</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>La apertura de sobres se realizará el día 14 de septiembre del 2026 a las 10:00 horas, en la sede municipal</t>
+          <t>Viernes 11 de Septiembre de 2026- a las 10:00 horas en la Sede Comunal de Comuna Distrito Sauce</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -985,7 +993,7 @@
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>El pliego será gratuito. El mismo se encontrará para su consulta y ent</t>
+          <t xml:space="preserve">sin costo. Solicitar en la Sede Comunal de Distrito Sauce Nogoya o al </t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
@@ -1005,7 +1013,7 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-ddc4dfb118d357f7</t>
+          <t>id-328f5a2f67c14702</t>
         </is>
       </c>
     </row>
@@ -1037,22 +1045,22 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>76/2026</t>
+          <t>77/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>ADQUICION DE CAMIONES COMPACTADORES DE CARGA TRASERA RSU</t>
+          <t>ADQUISICION DE CAMIONETAS</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>14-09-2026 08:00</t>
+          <t>11-09-2026 08:00</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1078,7 +1086,7 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-ccdfae2a7ede4696</t>
+          <t>id-dff70529581309e6</t>
         </is>
       </c>
     </row>
@@ -1095,12 +1103,12 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1110,22 +1118,22 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>014/2026</t>
+          <t>06/2026</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
+          <t>Transporte de dos mil metros cúbicos (2.000 m³) de ripio arcilloso destinados al mantenimiento y mejoramiento de caminos de la jurisdicción comunal de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>14 de septiembre de 2026 - Hora: 10:00</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1133,11 +1141,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
-        </is>
-      </c>
+      <c r="K9" s="4" t="inlineStr"/>
       <c r="L9" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1155,7 +1159,7 @@
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-9e58cc9ec0b69356</t>
+          <t>id-85e6cfd11c8a8889</t>
         </is>
       </c>
     </row>
@@ -1170,14 +1174,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>MUNICIPIO DE ORO VERDE</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1185,24 +1189,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>08/2026</t>
-        </is>
-      </c>
+      <c r="F10" s="4" t="inlineStr"/>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
+          <t>El procedimiento licitatorio regido por el presente pliego tiene por objeto la Licitación Pública N° 03/2026 para la venta de los siguientes bienes municipales: a) MINI RETRO DE TIRO: Marca RICHIGER, Serie A, N° 101. Modelo N° 186. Motor N° 991023899, C. V 7, 50, Modelo 7, 50 DB, RPM 1.500 b) COLECTIVO: Mercedes Benz, dominio UKZ353, modelo 1977 según lo que s e detalla en el Pliego de Bases y Condiciones que forma parte de la presente como Anexo I</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
+          <t>La apertura de sobres se realizará el día 14 de septiembre del 2026 a las 10:00 horas, en la sede municipal</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1210,21 +1210,29 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>El pliego será gratuito. El mismo se encontrará para su consulta y ent</t>
+        </is>
+      </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
+      <c r="M10" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-952aef4c115d8f12</t>
+          <t>id-ddc4dfb118d357f7</t>
         </is>
       </c>
     </row>
@@ -1239,39 +1247,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>27/2026</t>
+          <t>76/2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
+          <t>ADQUICION DE CAMIONES COMPACTADORES DE CARGA TRASERA RSU</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>16/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>16 de septiembre de 2026 - Hora: 10:00</t>
+          <t>14-09-2026 08:00</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1292,12 +1300,12 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-608017f47f903d65</t>
+          <t>id-ccdfae2a7ede4696</t>
         </is>
       </c>
     </row>
@@ -1312,14 +1320,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1329,22 +1337,22 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>06/26</t>
+          <t>014/2026</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en calle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
+          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1354,7 +1362,7 @@
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
+          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -1374,7 +1382,7 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-9dbdaa6090d92bd4</t>
+          <t>id-9e58cc9ec0b69356</t>
         </is>
       </c>
     </row>
@@ -1396,7 +1404,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SEGUÍ</t>
+          <t xml:space="preserve">ELECTRICA, CUBIERTA DE TECHO Y REFACCION DE BAÑOS ESCUELA Nº 1 “JOSE MARIA TEXIER” -SAN — </t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1406,30 +1414,34 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”. Apertura de Sobres 17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y entrega en Área de Suministro del Municipio, y también se podrá descargar en el Sitio Oficial Digital Municipal https://www.segui.gob.ar . Edgardo Muller, Presidente Municipal. ID:52321 - F.C. 04-00075716 3 v./03/09/2026</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “NUEVA INSTALACION ELECTRICA, CUBIERTA DE TECHO Y REFACCION DE BAÑOS ESCUELA Nº 1 “JOSE MARIA TEXIER” -SAN SALVADOR-DEPARTAMENTO SAN SALVADOR.”</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y</t>
+          <t>DE LAS OFERTAS: el día 15 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="K13" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1447,7 +1459,7 @@
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-90c3d1f38f49418a</t>
+          <t>id-fb80c8ade7a8651d</t>
         </is>
       </c>
     </row>
@@ -1462,14 +1474,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1479,22 +1491,22 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>015/2026</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
+          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1502,29 +1514,21 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
-        </is>
-      </c>
+      <c r="K14" s="4" t="inlineStr"/>
       <c r="L14" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M14" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
+      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-74dfdad7e5f9d048</t>
+          <t>id-952aef4c115d8f12</t>
         </is>
       </c>
     </row>
@@ -1539,14 +1543,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1556,22 +1560,22 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>27/2026</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
+          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
+          <t>16 de septiembre de 2026 - Hora: 10:00</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1585,15 +1589,19 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
+      <c r="M15" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-885d4847519dfd48</t>
+          <t>id-608017f47f903d65</t>
         </is>
       </c>
     </row>
@@ -1608,14 +1616,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1623,20 +1631,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>06/26</t>
+        </is>
+      </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
+          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>24 de SEPTIEMBRE de 2026</t>
+          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1646,7 +1658,7 @@
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>Sin Cargo</t>
+          <t>PESOS CINCUEN TA MIL ($ 50.000)</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">
@@ -1666,7 +1678,7 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-bc610b64999d147d</t>
+          <t>id-9dbdaa6090d92bd4</t>
         </is>
       </c>
     </row>
@@ -1688,7 +1700,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE — TERMINACION ESCUELA Nº 54</t>
+          <t>MUNICIPALIDAD DE SEGUÍ</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1698,22 +1710,22 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez realizado el depósito/transferenci</t>
+          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Usos Múltiples – Gimnasio Municipal”. Apertura de Sobres 17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y entrega en Área de Suministro del Municipio, y también se podrá descargar en el Sitio Oficial Digital Municipal https://www.segui.gob.ar . Edgardo Muller, Presidente Municipal. ID:52321 - F.C. 04-00075716 3 v./03/09/2026</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN N</t>
+          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1721,11 +1733,7 @@
           <t>17/09/2026</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t>Habilitación: Pesos Ochenta Mil con 0/100 - $ 80.000, 00 - Habilitació</t>
-        </is>
-      </c>
+      <c r="K17" s="4" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1743,7 +1751,7 @@
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-d97b43a99f1e1824</t>
+          <t>id-90c3d1f38f49418a</t>
         </is>
       </c>
     </row>
@@ -1758,14 +1766,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE — Y PUESTA EN VALOR – ESCUE</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1775,32 +1783,32 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>015/2026</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN</t>
+          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>Habilitación: Pesos Ciento Veinte Mil con 0/100 - $ 120.000, 00 - Habi</t>
+          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -1820,7 +1828,7 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-f8fab7a7b3a06a2d</t>
+          <t>id-74dfdad7e5f9d048</t>
         </is>
       </c>
     </row>
@@ -1842,7 +1850,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ — CONDARCO”</t>
+          <t>RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION — ELECTRICA-E</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1852,22 +1860,22 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>09/26</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1897,7 +1905,7 @@
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-6a4a84712fd41a03</t>
         </is>
       </c>
     </row>
@@ -1929,22 +1937,22 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
+          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1966,7 +1974,7 @@
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-885d4847519dfd48</t>
         </is>
       </c>
     </row>
@@ -1976,19 +1984,19 @@
           <t>08/09/2026</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1996,20 +2004,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>001-2026</t>
-        </is>
-      </c>
+      <c r="F21" s="4" t="inlineStr"/>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>L LAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr"/>
+          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>24 de SEPTIEMBRE de 2026</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2019,7 +2027,7 @@
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>Sin Cargo</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -2039,7 +2047,7 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-bc610b64999d147d</t>
         </is>
       </c>
     </row>
@@ -2049,19 +2057,19 @@
           <t>08/09/2026</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE — TERMINACION ESCUELA Nº 54</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2071,28 +2079,32 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr"/>
+          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez realizado el depósito/transferenci</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN N</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>s in cargo Consultas: comprascomuna6to@hotmail.com Celular: 3444- 4493</t>
+          <t>Habilitación: Pesos Ochenta Mil con 0/100 - $ 80.000, 00 - Habilitació</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr">
@@ -2112,7 +2124,7 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-511256e6329e386a</t>
+          <t>id-d97b43a99f1e1824</t>
         </is>
       </c>
     </row>
@@ -2122,19 +2134,19 @@
           <t>08/09/2026</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE — Y PUESTA EN VALOR – ESCUE</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2144,40 +2156,52 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr"/>
+          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K23" s="4" t="inlineStr"/>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>Habilitación: Pesos Ciento Veinte Mil con 0/100 - $ 120.000, 00 - Habi</t>
+        </is>
+      </c>
       <c r="L23" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
+      <c r="M23" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-f8fab7a7b3a06a2d</t>
         </is>
       </c>
     </row>
@@ -2187,19 +2211,19 @@
           <t>08/09/2026</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ — CONDARCO”</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2209,18 +2233,22 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr"/>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2228,21 +2256,29 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr"/>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L24" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
+      <c r="M24" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
@@ -2252,19 +2288,19 @@
           <t>08/09/2026</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2274,18 +2310,22 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr"/>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2302,12 +2342,12 @@
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
@@ -2322,14 +2362,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2339,18 +2379,18 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>L LAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2358,21 +2398,29 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr"/>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L26" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
+      <c r="M26" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
@@ -2387,14 +2435,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2404,18 +2452,18 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2423,21 +2471,29 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K27" s="4" t="inlineStr"/>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>s in cargo Consultas: comprascomuna6to@hotmail.com Celular: 3444- 4493</t>
+        </is>
+      </c>
       <c r="L27" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr"/>
+      <c r="M27" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2508,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
+      <c r="C28" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2467,16 +2523,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr"/>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>03/26</t>
+        </is>
+      </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2498,7 +2558,7 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2573,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="8" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2530,18 +2590,18 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>04/2025</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2563,7 +2623,7 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -2578,7 +2638,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr">
+      <c r="C30" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2595,18 +2655,18 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2628,7 +2688,7 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -2643,7 +2703,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2660,18 +2720,18 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2693,7 +2753,7 @@
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -2708,7 +2768,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr">
+      <c r="C32" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2725,18 +2785,18 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2758,7 +2818,7 @@
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -2773,35 +2833,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C33" s="8" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Concurso</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>01/26</t>
-        </is>
-      </c>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr"/>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2818,12 +2874,12 @@
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -2840,12 +2896,12 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Áridos</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2855,18 +2911,18 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>499/26</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA Nº 499/26: EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2883,12 +2939,12 @@
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-f53eab44dba8d43f</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
@@ -2903,35 +2959,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>235/26</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>Licitación Privada N° 235/26: reparación de cenefas en losas pórticos</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -2948,12 +3004,12 @@
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-22f9c51cdaebefb7</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
@@ -2968,14 +3024,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2985,18 +3041,18 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>498/26</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA N° 498/26: reparación de un tramo del cerramiento perimetral del Túnel Subfluvial</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3013,17 +3069,342 @@
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr">
         <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O36" s="4" t="inlineStr">
+        <is>
+          <t>id-07ddb93a12c5a870</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>IAPV (Vivienda)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>Concurso de Precio N° 02/2025</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr"/>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>Publicada 19/06/2025 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K37" s="4" t="inlineStr"/>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O37" s="4" t="inlineStr">
+        <is>
+          <t>id-7c1bf02160a66f67</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Concurso</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>01/26</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr"/>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K38" s="4" t="inlineStr"/>
+      <c r="L38" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="O38" s="4" t="inlineStr">
+        <is>
+          <t>id-9a16884dd5a64a49</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Áridos</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
           <t>Túnel Subfluvial</t>
         </is>
       </c>
-      <c r="O36" s="4" t="inlineStr">
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>499/26</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>LICITACIÓN PÚBLICA Nº 499/26: EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr"/>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K39" s="4" t="inlineStr"/>
+      <c r="L39" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Túnel Subfluvial</t>
+        </is>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>id-f53eab44dba8d43f</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Túnel Subfluvial</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Licitación Privada</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>235/26</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>Licitación Privada N° 235/26: reparación de cenefas en losas pórticos</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr"/>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K40" s="4" t="inlineStr"/>
+      <c r="L40" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Túnel Subfluvial</t>
+        </is>
+      </c>
+      <c r="O40" s="4" t="inlineStr">
+        <is>
+          <t>id-22f9c51cdaebefb7</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Túnel Subfluvial</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>498/26</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>LICITACIÓN PÚBLICA N° 498/26: reparación de un tramo del cerramiento perimetral del Túnel Subfluvial</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr"/>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K41" s="4" t="inlineStr"/>
+      <c r="L41" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Túnel Subfluvial</t>
+        </is>
+      </c>
+      <c r="O41" s="4" t="inlineStr">
         <is>
           <t>id-46d81e3efd2ae483</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O36"/>
+  <autoFilter ref="A1:O41"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3042,42 +3423,52 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId63"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Corregir el organismo en los avisos del Boletín
El título de la obra viene en mayúsculas igual que el nombre del organismo, así
que se colaba en su lugar ('CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS').
Ahora sólo se acepta una línea que empiece como organismo (municipalidad,
comuna, gobierno, ente, comisión...) o que sea una localidad corta que no
mencione trabajos de obra.
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -658,7 +658,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CHAJARI — APERTURA: 08 DE SEPTIEMBRE DE 2026 - HORA: 10:00 (DIEZ) - SI ES</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1404,7 +1404,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">ELECTRICA, CUBIERTA DE TECHO Y REFACCION DE BAÑOS ESCUELA Nº 1 “JOSE MARIA TEXIER” -SAN — </t>
+          <t>MINISTERIO DE PLANEAMIENTO E INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1850,7 +1850,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION — ELECTRICA-E</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE — TERMINACION ESCUELA Nº 54</t>
+          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2146,7 +2146,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE — Y PUESTA EN VALOR – ESCUE</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ — CONDARCO”</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">

</xml_diff>

<commit_message>
Los enlaces del Boletín abren en la página del aviso
El boletín tiene ~100 páginas y había que buscar el aviso a mano (el de Villa
Elisa estaba en la 75). Ahora se intercala una marca invisible por página al
extraer el texto y el enlace lleva #page=N; la planilla muestra 'ver pág. 75'.

La marca va al principio de cada página, así que para un aviso que entra entero
en una sola hay que mirar la marca ANTERIOR, no las de adentro: mirando sólo
adentro se detectaban 11 de 27; ahora 25 de 27.
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -62,12 +62,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:O40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -566,7 +566,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -643,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -653,37 +653,37 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
+          <t>FEDERACION — COMUNA DE SAN PEDRO -- DEPARTAMENTO DE FEDERACIÓN</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Licitacion Publica</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>013/2026</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – hierro y otros – que serán destinados a la construcción de viviendas que se llevarán a cabo en el marco del Plan Construir Futuro 7</t>
+          <t>“PROVISION RIPIO SELECCIONADO EN ORIGEN Y ENTREGADO SOBRE TRANSPORTE”</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>08 DE SEPTIEMBRE DE 2026 - HORA: 10:00 (DIEZ)</t>
+          <t>09 de Septiembre de 2026 - 10:00 hs</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>$ 100.000,00.- (PESOS CIEN MIL CON 00/100) PRESUPUESTO OFICIAL ESTIMAD</t>
+          <t>Sin costo</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
@@ -713,14 +713,14 @@
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>id-2ac90305e5165aad</t>
+          <t>id-719cc55444d8579b</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -728,14 +728,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>FEDERACION — COMUNA DE SAN PEDRO -- DEPARTAMENTO DE FEDERACIÓN</t>
+          <t>CONCORDIA — MUNICIPALIDAD DE PUERTO YERUA</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -745,22 +745,22 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>1/2026</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>“PROVISION RIPIO SELECCIONADO EN ORIGEN Y ENTREGADO SOBRE TRANSPORTE”</t>
+          <t>Adquisición de una motoniveladora 0 Km</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>09 de Septiembre de 2026 - 10:00 hs</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -768,11 +768,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>Sin costo</t>
-        </is>
-      </c>
+      <c r="K4" s="4" t="inlineStr"/>
       <c r="L4" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -790,14 +786,14 @@
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>id-719cc55444d8579b</t>
+          <t>id-61b6e4f9568150b0</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -805,14 +801,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>CONCORDIA — MUNICIPALIDAD DE PUERTO YERUA</t>
+          <t>ENTE INTERPROVINCIAL TUNEL SUBFLUVIAL RAUL URANGA -- CARLOS S. BEGNIS</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -820,14 +816,10 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>1/2026</t>
-        </is>
-      </c>
+      <c r="F5" s="4" t="inlineStr"/>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de una motoniveladora 0 Km</t>
+          <t>EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -845,7 +837,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>GRATUITO FECHA DE APERTURA: 10/09/2026</t>
+        </is>
+      </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -863,14 +859,14 @@
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-61b6e4f9568150b0</t>
+          <t>id-439ddd7aaa7f7b3e</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -878,14 +874,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ENTE INTERPROVINCIAL TUNEL SUBFLUVIAL RAUL URANGA -- CARLOS S. BEGNIS</t>
+          <t>NOGOYA — COMUNA DISTRITO SAUCE -- NOGOYA</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -893,20 +889,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr"/>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>1/26</t>
+        </is>
+      </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
+          <t>Convocar para la adquisi ción de un Tractor agrícola 0 km, con las siguientes características técnicas: potencia de motor de 130 a 150 HP; doble Tracción, 6 (seis) cilindros; y demás especificación que se encuentran en el pliego de Especificaciones Técnicas</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>Viernes 11 de Septiembre de 2026- a las 10:00 horas en la Sede Comunal de Comuna Distrito Sauce</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>GRATUITO FECHA DE APERTURA: 10/09/2026</t>
+          <t xml:space="preserve">sin costo. Solicitar en la Sede Comunal de Distrito Sauce Nogoya o al </t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
@@ -936,14 +936,14 @@
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-439ddd7aaa7f7b3e</t>
+          <t>id-328f5a2f67c14702</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -958,22 +958,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>NOGOYA — COMUNA DISTRITO SAUCE -- NOGOYA</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>1/26</t>
+          <t>77/2026</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Convocar para la adquisi ción de un Tractor agrícola 0 km, con las siguientes características técnicas: potencia de motor de 130 a 150 HP; doble Tracción, 6 (seis) cilindros; y demás especificación que se encuentran en el pliego de Especificaciones Técnicas</t>
+          <t>ADQUISICION DE CAMIONETAS</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -983,7 +983,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Viernes 11 de Septiembre de 2026- a las 10:00 horas en la Sede Comunal de Comuna Distrito Sauce</t>
+          <t>11-09-2026 08:00</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -991,11 +991,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sin costo. Solicitar en la Sede Comunal de Distrito Sauce Nogoya o al </t>
-        </is>
-      </c>
+      <c r="K7" s="4" t="inlineStr"/>
       <c r="L7" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1008,19 +1004,19 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-328f5a2f67c14702</t>
+          <t>id-dff70529581309e6</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1028,39 +1024,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>77/2026</t>
+          <t>06/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICION DE CAMIONETAS</t>
+          <t>Transporte de dos mil metros cúbicos (2.000 m³) de ripio arcilloso destinados al mantenimiento y mejoramiento de caminos de la jurisdicción comunal de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>11-09-2026 08:00</t>
+          <t>14 de septiembre de 2026 - Hora: 10:00</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1081,19 +1077,19 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-dff70529581309e6</t>
+          <t>id-85e6cfd11c8a8889</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1101,14 +1097,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>MUNICIPIO DE ORO VERDE</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1116,14 +1112,10 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>06/2026</t>
-        </is>
-      </c>
+      <c r="F9" s="4" t="inlineStr"/>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Transporte de dos mil metros cúbicos (2.000 m³) de ripio arcilloso destinados al mantenimiento y mejoramiento de caminos de la jurisdicción comunal de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>El procedimiento licitatorio regido por el presente pliego tiene por objeto la Licitación Pública N° 03/2026 para la venta de los siguientes bienes municipales: a) MINI RETRO DE TIRO: Marca RICHIGER, Serie A, N° 101. Modelo N° 186. Motor N° 991023899, C. V 7, 50, Modelo 7, 50 DB, RPM 1.500 b) COLECTIVO: Mercedes Benz, dominio UKZ353, modelo 1977 según lo que s e detalla en el Pliego de Bases y Condiciones que forma parte de la presente como Anexo I</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1133,7 +1125,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>14 de septiembre de 2026 - Hora: 10:00</t>
+          <t>La apertura de sobres se realizará el día 14 de septiembre del 2026 a las 10:00 horas, en la sede municipal</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1141,7 +1133,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr"/>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>El pliego será gratuito. El mismo se encontrará para su consulta y ent</t>
+        </is>
+      </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1159,14 +1155,14 @@
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-85e6cfd11c8a8889</t>
+          <t>id-ddc4dfb118d357f7</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1181,18 +1177,22 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE ORO VERDE</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr"/>
+          <t>LICITACIÓN PÚBLICA</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>76/2026</t>
+        </is>
+      </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>El procedimiento licitatorio regido por el presente pliego tiene por objeto la Licitación Pública N° 03/2026 para la venta de los siguientes bienes municipales: a) MINI RETRO DE TIRO: Marca RICHIGER, Serie A, N° 101. Modelo N° 186. Motor N° 991023899, C. V 7, 50, Modelo 7, 50 DB, RPM 1.500 b) COLECTIVO: Mercedes Benz, dominio UKZ353, modelo 1977 según lo que s e detalla en el Pliego de Bases y Condiciones que forma parte de la presente como Anexo I</t>
+          <t>ADQUICION DE CAMIONES COMPACTADORES DE CARGA TRASERA RSU</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>La apertura de sobres se realizará el día 14 de septiembre del 2026 a las 10:00 horas, en la sede municipal</t>
+          <t>14-09-2026 08:00</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1210,11 +1210,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>El pliego será gratuito. El mismo se encontrará para su consulta y ent</t>
-        </is>
-      </c>
+      <c r="K10" s="4" t="inlineStr"/>
       <c r="L10" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1227,19 +1223,19 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-ddc4dfb118d357f7</t>
+          <t>id-ccdfae2a7ede4696</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1247,39 +1243,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>76/2026</t>
+          <t>014/2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>ADQUICION DE CAMIONES COMPACTADORES DE CARGA TRASERA RSU</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>14-09-2026 08:00</t>
+          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1287,7 +1283,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr"/>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
+        </is>
+      </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1300,19 +1300,19 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-ccdfae2a7ede4696</t>
+          <t>id-9e58cc9ec0b69356</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1320,14 +1320,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
+          <t>MINISTERIO DE PLANEAMIENTO E INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1337,12 +1337,12 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>014/2026</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “NUEVA INSTALACION ELECTRICA, CUBIERTA DE TECHO Y REFACCION DE BAÑOS ESCUELA Nº 1 “JOSE MARIA TEXIER” -SAN SALVADOR-DEPARTAMENTO SAN SALVADOR.”</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>DE LAS OFERTAS: el día 15 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -1382,14 +1382,14 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-9e58cc9ec0b69356</t>
+          <t>id-fb80c8ade7a8651d</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1404,7 +1404,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO E INFRAESTRUCTURA</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1414,12 +1414,12 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “NUEVA INSTALACION ELECTRICA, CUBIERTA DE TECHO Y REFACCION DE BAÑOS ESCUELA Nº 1 “JOSE MARIA TEXIER” -SAN SALVADOR-DEPARTAMENTO SAN SALVADOR.”</t>
+          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 15 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1437,36 +1437,28 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K13" s="4" t="inlineStr"/>
       <c r="L13" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M13" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
+      <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-fb80c8ade7a8651d</t>
+          <t>id-952aef4c115d8f12</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1474,14 +1466,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1491,22 +1483,22 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>27/2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
+          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
+          <t>16 de septiembre de 2026 - Hora: 10:00</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1520,22 +1512,26 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
+      <c r="M14" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-952aef4c115d8f12</t>
+          <t>id-608017f47f903d65</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1543,14 +1539,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
+          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1560,22 +1556,22 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>27/2026</t>
+          <t>06/26</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
+          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>16/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>16 de septiembre de 2026 - Hora: 10:00</t>
+          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1583,7 +1579,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
+        </is>
+      </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1601,14 +1601,14 @@
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-608017f47f903d65</t>
+          <t>id-9dbdaa6090d92bd4</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
+          <t>MUNICIPALIDAD DE SEGUÍ</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1633,12 +1633,12 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>06/26</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
+          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”. Apertura de Sobres 17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y entrega en Área de Suministro del Municipio, y también se podrá descargar en el Sitio Oficial Digital Municipal https://www.segui.gob.ar . Edgardo Muller, Presidente Municipal. ID:52321 - F.C. 04-00075716 3 v./03/09/2026</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1648,19 +1648,15 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
+          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
-        </is>
-      </c>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1678,14 +1674,14 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-9dbdaa6090d92bd4</t>
+          <t>id-90c3d1f38f49418a</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1693,14 +1689,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SEGUÍ</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1710,30 +1706,34 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>015/2026</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”. Apertura de Sobres 17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y entrega en Área de Suministro del Municipio, y también se podrá descargar en el Sitio Oficial Digital Municipal https://www.segui.gob.ar . Edgardo Muller, Presidente Municipal. ID:52321 - F.C. 04-00075716 3 v./03/09/2026</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y</t>
+          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
+        </is>
+      </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1751,14 +1751,14 @@
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-90c3d1f38f49418a</t>
+          <t>id-74dfdad7e5f9d048</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1766,14 +1766,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1783,12 +1783,12 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>015/2026</t>
+          <t>09/26</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -1828,14 +1828,14 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-74dfdad7e5f9d048</t>
+          <t>id-6a4a84712fd41a03</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1850,7 +1850,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1860,12 +1860,12 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>09/26</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
+          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1883,36 +1883,28 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K19" s="4" t="inlineStr"/>
       <c r="L19" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M19" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
+      <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-6a4a84712fd41a03</t>
+          <t>id-885d4847519dfd48</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1920,14 +1912,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1935,24 +1927,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>09/2026</t>
-        </is>
-      </c>
+      <c r="F20" s="4" t="inlineStr"/>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
+          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
+          <t>24 de SEPTIEMBRE de 2026</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1960,28 +1948,36 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>Sin Cargo</t>
+        </is>
+      </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
+      <c r="M20" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-885d4847519dfd48</t>
+          <t>id-bc610b64999d147d</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1989,14 +1985,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2004,10 +2000,14 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr"/>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>10/2026</t>
+        </is>
+      </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
+          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez realizado el depósito/transferenci</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -2017,17 +2017,17 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>24 de SEPTIEMBRE de 2026</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN N</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>Sin Cargo</t>
+          <t>Habilitación: Pesos Ochenta Mil con 0/100 - $ 80.000, 00 - Habilitació</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -2047,14 +2047,14 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-bc610b64999d147d</t>
+          <t>id-d97b43a99f1e1824</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2079,12 +2079,12 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez realizado el depósito/transferenci</t>
+          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -2094,7 +2094,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN N</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2104,7 +2104,7 @@
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>Habilitación: Pesos Ochenta Mil con 0/100 - $ 80.000, 00 - Habilitació</t>
+          <t>Habilitación: Pesos Ciento Veinte Mil con 0/100 - $ 120.000, 00 - Habi</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr">
@@ -2124,14 +2124,14 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-d97b43a99f1e1824</t>
+          <t>id-f8fab7a7b3a06a2d</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2146,7 +2146,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2156,32 +2156,32 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>Habilitación: Pesos Ciento Veinte Mil con 0/100 - $ 120.000, 00 - Habi</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
@@ -2201,14 +2201,14 @@
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-f8fab7a7b3a06a2d</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2233,12 +2233,12 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -2248,7 +2248,7 @@
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2256,41 +2256,33 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K24" s="4" t="inlineStr"/>
       <c r="L24" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M24" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
+      <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -2300,7 +2292,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2310,22 +2302,18 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
+          <t>L LAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2333,28 +2321,36 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr"/>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L25" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
+      <c r="M25" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2362,14 +2358,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2379,12 +2375,12 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>L LAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
@@ -2400,7 +2396,7 @@
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>s in cargo Consultas: comprascomuna6to@hotmail.com Celular: 3444- 4493</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr">
@@ -2420,14 +2416,14 @@
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2435,14 +2431,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2452,18 +2448,18 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2471,36 +2467,28 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K27" s="4" t="inlineStr">
-        <is>
-          <t>s in cargo Consultas: comprascomuna6to@hotmail.com Celular: 3444- 4493</t>
-        </is>
-      </c>
+      <c r="K27" s="4" t="inlineStr"/>
       <c r="L27" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M27" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
+      <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-511256e6329e386a</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2508,7 +2496,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C28" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2525,18 +2513,18 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2558,14 +2546,14 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2573,7 +2561,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C29" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2590,18 +2578,18 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2623,14 +2611,14 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2638,7 +2626,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2655,18 +2643,18 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2688,14 +2676,14 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2703,7 +2691,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2720,18 +2708,18 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2753,14 +2741,14 @@
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2768,7 +2756,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
+      <c r="C32" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2783,20 +2771,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>06/2025</t>
-        </is>
-      </c>
+      <c r="F32" s="4" t="inlineStr"/>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2818,14 +2802,14 @@
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2833,7 +2817,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2848,16 +2832,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr"/>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2879,14 +2867,14 @@
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2894,7 +2882,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C34" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2911,18 +2899,18 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>04/2025</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2944,14 +2932,14 @@
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2959,7 +2947,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="C35" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2976,18 +2964,18 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3009,14 +2997,14 @@
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3024,7 +3012,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
+      <c r="C36" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -3046,13 +3034,13 @@
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3074,14 +3062,14 @@
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3089,35 +3077,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
+      <c r="C37" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>01/26</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3134,19 +3122,19 @@
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3156,27 +3144,27 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>Túnel Subfluvial</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>499/26</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>LICITACIÓN PÚBLICA Nº 499/26: EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
@@ -3199,19 +3187,19 @@
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>Túnel Subfluvial</t>
         </is>
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-f53eab44dba8d43f</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3219,9 +3207,9 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -3231,17 +3219,17 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación Privada</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>499/26</t>
+          <t>235/26</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA Nº 499/26: EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
+          <t>Licitación Privada N° 235/26: reparación de cenefas en losas pórticos</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
@@ -3269,14 +3257,14 @@
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-f53eab44dba8d43f</t>
+          <t>id-22f9c51cdaebefb7</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3296,17 +3284,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>235/26</t>
+          <t>498/26</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>Licitación Privada N° 235/26: reparación de cenefas en losas pórticos</t>
+          <t>LICITACIÓN PÚBLICA N° 498/26: reparación de un tramo del cerramiento perimetral del Túnel Subfluvial</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
@@ -3334,77 +3322,12 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-22f9c51cdaebefb7</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>08/09/2026</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C41" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Túnel Subfluvial</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>498/26</t>
-        </is>
-      </c>
-      <c r="G41" s="5" t="inlineStr">
-        <is>
-          <t>LICITACIÓN PÚBLICA N° 498/26: reparación de un tramo del cerramiento perimetral del Túnel Subfluvial</t>
-        </is>
-      </c>
-      <c r="H41" s="4" t="inlineStr"/>
-      <c r="I41" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J41" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K41" s="4" t="inlineStr"/>
-      <c r="L41" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>Túnel Subfluvial</t>
-        </is>
-      </c>
-      <c r="O41" s="4" t="inlineStr">
-        <is>
           <t>id-46d81e3efd2ae483</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O41"/>
+  <autoFilter ref="A1:O40"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3429,8 +3352,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId28"/>
@@ -3440,8 +3363,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId39"/>
@@ -3449,26 +3372,24 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId61"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fuentes que pasó el ingeniero + parser de CAFESG
- URLs corregidas: Crespo (la anterior mostraba 2016) y Oro Verde (la anterior
  se colgaba). Ambas vuelven a estar activas.
- Nuevas: CAFESG, San Benito, Aldea Brasilera, Poder Judicial e IAPSER.
- Parser propio para CAFESG: cada llamado tiene su página y el listado indica el
  estado, así que se filtran los que siguen abiertos (3 de 72). Aporta
  licitaciones PRIVADAS que no aparecen en el Boletín.
- La planilla suma 'Probar conexión', que dice si puede leer el listado y el
  estado de las fuentes, y muestra la versión del script.
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O40"/>
+  <dimension ref="A1:O44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Transporte de dos mil metros cúbicos (2.000 m³) de ripio arcilloso destinados al mantenimiento y mejoramiento de caminos de la jurisdicción comunal de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>Transporte de dos mil metros cúbicos (2.000 m³) de ripio arcilloso destinados al mantenimiento y mejoramiento de caminos de la jurisdicción comunal de acuerdo a los Pliegos de Bases, C ondiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -1243,14 +1243,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
+          <t>MUNICIPALIDAD DE HERRERA — DPTO. URUGUAY, ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1260,12 +1260,12 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>014/2026</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
+          <t>Adquisición de vehículo 0 km destinado al traslado de personas tipo van, con capacidad para 11 plazas (1 conductor + 10 pasajeros), motorización a nafta/diesel, según pliego de espec ificaciones técnicas</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>DE LAS OFERTAS: el día 15/09/2026, a las 11:00 hs. en el Edificio Municipal de Herrera, sito en Av. H. Bozzolo, Nº 165,</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-9e58cc9ec0b69356</t>
+          <t>id-28313c7a9524d0ee</t>
         </is>
       </c>
     </row>
@@ -1320,14 +1320,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO E INFRAESTRUCTURA</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1337,12 +1337,12 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>014/2026</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “NUEVA INSTALACION ELECTRICA, CUBIERTA DE TECHO Y REFACCION DE BAÑOS ESCUELA Nº 1 “JOSE MARIA TEXIER” -SAN SALVADOR-DEPARTAMENTO SAN SALVADOR.”</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 15 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-fb80c8ade7a8651d</t>
+          <t>id-9e58cc9ec0b69356</t>
         </is>
       </c>
     </row>
@@ -1404,7 +1404,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>MINISTERIO DE PLANEAMIENTO E INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1414,12 +1414,12 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “NUEVA INSTALACION ELECTRICA, CUBIERTA DE TECHO Y REFACCION DE BAÑOS ESCUELA Nº 1 “JOSE MARIA TEXIER” -SAN SALVADOR-DEPARTAMENTO SAN SALVADOR.”</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
+          <t>DE LAS OFERTAS: el día 15 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1437,21 +1437,29 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr"/>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
+      <c r="M13" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-952aef4c115d8f12</t>
+          <t>id-fb80c8ade7a8651d</t>
         </is>
       </c>
     </row>
@@ -1466,14 +1474,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1483,22 +1491,22 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>27/2026</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
+          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>16/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>16 de septiembre de 2026 - Hora: 10:00</t>
+          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1512,19 +1520,15 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M14" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
+      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-608017f47f903d65</t>
+          <t>id-952aef4c115d8f12</t>
         </is>
       </c>
     </row>
@@ -1539,14 +1543,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
+          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1556,22 +1560,22 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>06/26</t>
+          <t>27/2026</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
+          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
+          <t>16 de septiembre de 2026 - Hora: 10:00</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1579,11 +1583,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
-        </is>
-      </c>
+      <c r="K15" s="4" t="inlineStr"/>
       <c r="L15" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-9dbdaa6090d92bd4</t>
+          <t>id-608017f47f903d65</t>
         </is>
       </c>
     </row>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SEGUÍ</t>
+          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1633,12 +1633,12 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>06/26</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”. Apertura de Sobres 17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y entrega en Área de Suministro del Municipio, y también se podrá descargar en el Sitio Oficial Digital Municipal https://www.segui.gob.ar . Edgardo Muller, Presidente Municipal. ID:52321 - F.C. 04-00075716 3 v./03/09/2026</t>
+          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1648,15 +1648,19 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y</t>
+          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
+        </is>
+      </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1674,7 +1678,7 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-90c3d1f38f49418a</t>
+          <t>id-9dbdaa6090d92bd4</t>
         </is>
       </c>
     </row>
@@ -1689,14 +1693,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
+          <t>MUNICIPALIDAD DE SEGUÍ</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1706,34 +1710,30 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>015/2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
+          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”. Apertura de Sobres 17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y entrega en Área de Suministro del Municipio, y también se podrá descargar en el Sitio Oficial Digital Municipal https://www.segui.gob.ar . Edgardo Muller, Presidente Municipal. ID:52321 - F.C. 04-00075716 3 v./03/09/2026</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
-        </is>
-      </c>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1751,7 +1751,7 @@
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-74dfdad7e5f9d048</t>
+          <t>id-90c3d1f38f49418a</t>
         </is>
       </c>
     </row>
@@ -1766,14 +1766,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1783,12 +1783,12 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>09/26</t>
+          <t>015/2026</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -1828,7 +1828,7 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-6a4a84712fd41a03</t>
+          <t>id-74dfdad7e5f9d048</t>
         </is>
       </c>
     </row>
@@ -1850,7 +1850,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1860,12 +1860,12 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>09/26</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
+          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1883,21 +1883,29 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr"/>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L19" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr"/>
+      <c r="M19" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-885d4847519dfd48</t>
+          <t>id-6a4a84712fd41a03</t>
         </is>
       </c>
     </row>
@@ -1912,14 +1920,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1927,20 +1935,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr"/>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>09/2026</t>
+        </is>
+      </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
+          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>24 de SEPTIEMBRE de 2026</t>
+          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1948,29 +1960,21 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K20" s="4" t="inlineStr">
-        <is>
-          <t>Sin Cargo</t>
-        </is>
-      </c>
+      <c r="K20" s="4" t="inlineStr"/>
       <c r="L20" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M20" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
+      <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-bc610b64999d147d</t>
+          <t>id-885d4847519dfd48</t>
         </is>
       </c>
     </row>
@@ -1985,14 +1989,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2000,14 +2004,10 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>10/2026</t>
-        </is>
-      </c>
+      <c r="F21" s="4" t="inlineStr"/>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez realizado el depósito/transferenci</t>
+          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -2017,17 +2017,17 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN N</t>
+          <t>24 de SEPTIEMBRE de 2026</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>Habilitación: Pesos Ochenta Mil con 0/100 - $ 80.000, 00 - Habilitació</t>
+          <t>Sin Cargo</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-d97b43a99f1e1824</t>
+          <t>id-bc610b64999d147d</t>
         </is>
       </c>
     </row>
@@ -2069,7 +2069,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2079,12 +2079,12 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez</t>
+          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez realizado el depósito/transferenci</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -2094,7 +2094,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN N</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2104,7 +2104,7 @@
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>Habilitación: Pesos Ciento Veinte Mil con 0/100 - $ 120.000, 00 - Habi</t>
+          <t>Habilitación: Pesos Ochenta Mil con 0/100 - $ 80.000, 00 - Habilitació</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr">
@@ -2124,7 +2124,7 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-f8fab7a7b3a06a2d</t>
+          <t>id-d97b43a99f1e1824</t>
         </is>
       </c>
     </row>
@@ -2146,7 +2146,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2156,32 +2156,32 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>Habilitación: Pesos Ciento Veinte Mil con 0/100 - $ 120.000, 00 - Habi</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-f8fab7a7b3a06a2d</t>
         </is>
       </c>
     </row>
@@ -2223,7 +2223,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2233,12 +2233,12 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -2248,7 +2248,7 @@
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2256,21 +2256,29 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr"/>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L24" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
+      <c r="M24" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
@@ -2280,9 +2288,9 @@
           <t>09/09/2026</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -2292,7 +2300,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2302,18 +2310,22 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>L LAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr"/>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2321,29 +2333,21 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K25" s="4" t="inlineStr"/>
       <c r="L25" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M25" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
+      <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
@@ -2358,14 +2362,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2375,18 +2379,18 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2396,7 +2400,7 @@
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>s in cargo Consultas: comprascomuna6to@hotmail.com Celular: 3444- 4493</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr">
@@ -2416,7 +2420,7 @@
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-511256e6329e386a</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
@@ -2431,14 +2435,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2448,18 +2452,18 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2467,21 +2471,29 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K27" s="4" t="inlineStr"/>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>s in cargo Consultas: comprascomuna6to@hotmail.com Celular: 3444- 4493</t>
+        </is>
+      </c>
       <c r="L27" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr"/>
+      <c r="M27" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
@@ -2513,18 +2525,18 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2546,7 +2558,7 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
@@ -2578,18 +2590,18 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2611,7 +2623,7 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -2643,18 +2655,18 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2676,7 +2688,7 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -2708,18 +2720,18 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2741,7 +2753,7 @@
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -2771,16 +2783,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr"/>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2802,7 +2818,7 @@
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -2832,20 +2848,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>04/2025</t>
-        </is>
-      </c>
+      <c r="F33" s="4" t="inlineStr"/>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2867,7 +2879,7 @@
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -2899,18 +2911,18 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2932,7 +2944,7 @@
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
@@ -2964,18 +2976,18 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -2997,7 +3009,7 @@
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
@@ -3034,13 +3046,13 @@
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3062,7 +3074,7 @@
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
@@ -3084,28 +3096,28 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3122,12 +3134,12 @@
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
@@ -3142,29 +3154,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>499/26</t>
+          <t>01/26</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA Nº 499/26: EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
@@ -3187,12 +3199,12 @@
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-f53eab44dba8d43f</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
@@ -3207,9 +3219,9 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C39" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -3219,17 +3231,17 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>235/26</t>
+          <t>499/26</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>Licitación Privada N° 235/26: reparación de cenefas en losas pórticos</t>
+          <t>LICITACIÓN PÚBLICA Nº 499/26: EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
@@ -3257,7 +3269,7 @@
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-22f9c51cdaebefb7</t>
+          <t>id-f53eab44dba8d43f</t>
         </is>
       </c>
     </row>
@@ -3284,17 +3296,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación Privada</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>498/26</t>
+          <t>235/26</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA N° 498/26: reparación de un tramo del cerramiento perimetral del Túnel Subfluvial</t>
+          <t>Licitación Privada N° 235/26: reparación de cenefas en losas pórticos</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
@@ -3322,12 +3334,272 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
+          <t>id-22f9c51cdaebefb7</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Túnel Subfluvial</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>498/26</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>LICITACIÓN PÚBLICA N° 498/26: reparación de un tramo del cerramiento perimetral del Túnel Subfluvial</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr"/>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K41" s="4" t="inlineStr"/>
+      <c r="L41" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Túnel Subfluvial</t>
+        </is>
+      </c>
+      <c r="O41" s="4" t="inlineStr">
+        <is>
           <t>id-46d81e3efd2ae483</t>
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>10-2026</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr"/>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego — figura como Pendiente</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr"/>
+      <c r="L42" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="O42" s="4" t="inlineStr">
+        <is>
+          <t>id-bdd0abb0374c3f42</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>09-2026</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr"/>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego — figura como Pendiente</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr"/>
+      <c r="L43" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="O43" s="4" t="inlineStr">
+        <is>
+          <t>id-42c411be9946d956</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Licitación Privada</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>04-2026</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr"/>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego — figura como Pendiente</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K44" s="4" t="inlineStr"/>
+      <c r="L44" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="O44" s="4" t="inlineStr">
+        <is>
+          <t>id-023b6b75e7014a9c</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O40"/>
+  <autoFilter ref="A1:O44"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3352,8 +3624,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId28"/>
@@ -3363,8 +3635,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId39"/>
@@ -3372,24 +3644,29 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId66"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Poder Judicial andando, lectura de tablas y rubro Materiales
- El Poder Judicial titula 'Solicitud de Cotización Nº 225/26', que no estaba
  entre los disparadores: devolvía 0 y ahora trae 6.
- El parser genérico lee tablas de licitaciones (Crespo publica así) y prioriza
  títulos de artículos antes que líneas sueltas de texto. Crespo pasó de 0 a 5,
  con número, apertura y costo de pliego.
- Rubro MATERIALES: 'Adquisición de hormigón elaborado, malla sima y hierro' se
  estaba DESCARTANDO por no tener ninguna palabra de las listas, siendo del
  rubro. Recupera 5 licitaciones, entre ellas Urdinarrain (300 m³ de hormigón).
- Se descartan las ventas y remates de bienes del municipio: son al revés, el
  municipio vende, no compra.
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -43,7 +43,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -75,6 +75,11 @@
         <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6D9F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -88,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -101,6 +106,7 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -466,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O44"/>
+  <dimension ref="A1:O46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1104,18 +1110,22 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE ORO VERDE</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr"/>
+          <t>LICITACIÓN PÚBLICA</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>76/2026</t>
+        </is>
+      </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>El procedimiento licitatorio regido por el presente pliego tiene por objeto la Licitación Pública N° 03/2026 para la venta de los siguientes bienes municipales: a) MINI RETRO DE TIRO: Marca RICHIGER, Serie A, N° 101. Modelo N° 186. Motor N° 991023899, C. V 7, 50, Modelo 7, 50 DB, RPM 1.500 b) COLECTIVO: Mercedes Benz, dominio UKZ353, modelo 1977 según lo que s e detalla en el Pliego de Bases y Condiciones que forma parte de la presente como Anexo I</t>
+          <t>ADQUICION DE CAMIONES COMPACTADORES DE CARGA TRASERA RSU</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1125,7 +1135,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>La apertura de sobres se realizará el día 14 de septiembre del 2026 a las 10:00 horas, en la sede municipal</t>
+          <t>14-09-2026 08:00</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1133,11 +1143,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>El pliego será gratuito. El mismo se encontrará para su consulta y ent</t>
-        </is>
-      </c>
+      <c r="K9" s="4" t="inlineStr"/>
       <c r="L9" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1150,12 +1156,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-ddc4dfb118d357f7</t>
+          <t>id-ccdfae2a7ede4696</t>
         </is>
       </c>
     </row>
@@ -1177,32 +1183,32 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>MUNICIPALIDAD DE HERRERA — DPTO. URUGUAY, ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>76/2026</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>ADQUICION DE CAMIONES COMPACTADORES DE CARGA TRASERA RSU</t>
+          <t>Adquisición de vehículo 0 km destinado al traslado de personas tipo van, con capacidad para 11 plazas (1 conductor + 10 pasajeros), motorización a nafta/diesel, según pliego de espec ificaciones técnicas</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>14-09-2026 08:00</t>
+          <t>DE LAS OFERTAS: el día 15/09/2026, a las 11:00 hs. en el Edificio Municipal de Herrera, sito en Av. H. Bozzolo, Nº 165,</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1210,7 +1216,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1223,12 +1233,12 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-ccdfae2a7ede4696</t>
+          <t>id-28313c7a9524d0ee</t>
         </is>
       </c>
     </row>
@@ -1243,14 +1253,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE HERRERA — DPTO. URUGUAY, ENTRE RÍOS</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1260,12 +1270,12 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>014/2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de vehículo 0 km destinado al traslado de personas tipo van, con capacidad para 11 plazas (1 conductor + 10 pasajeros), motorización a nafta/diesel, según pliego de espec ificaciones técnicas</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1275,7 +1285,7 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 15/09/2026, a las 11:00 hs. en el Edificio Municipal de Herrera, sito en Av. H. Bozzolo, Nº 165,</t>
+          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1285,7 +1295,7 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -1305,7 +1315,7 @@
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-28313c7a9524d0ee</t>
+          <t>id-9e58cc9ec0b69356</t>
         </is>
       </c>
     </row>
@@ -1320,14 +1330,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
+          <t>MINISTERIO DE PLANEAMIENTO E INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1337,12 +1347,12 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>014/2026</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “NUEVA INSTALACION ELECTRICA, CUBIERTA DE TECHO Y REFACCION DE BAÑOS ESCUELA Nº 1 “JOSE MARIA TEXIER” -SAN SALVADOR-DEPARTAMENTO SAN SALVADOR.”</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1352,7 +1362,7 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>DE LAS OFERTAS: el día 15 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1362,7 +1372,7 @@
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -1382,7 +1392,7 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-9e58cc9ec0b69356</t>
+          <t>id-fb80c8ade7a8651d</t>
         </is>
       </c>
     </row>
@@ -1404,7 +1414,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO E INFRAESTRUCTURA</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1414,12 +1424,12 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “NUEVA INSTALACION ELECTRICA, CUBIERTA DE TECHO Y REFACCION DE BAÑOS ESCUELA Nº 1 “JOSE MARIA TEXIER” -SAN SALVADOR-DEPARTAMENTO SAN SALVADOR.”</t>
+          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1429,7 +1439,7 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 15 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1437,29 +1447,21 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K13" s="4" t="inlineStr"/>
       <c r="L13" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M13" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
+      <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-fb80c8ade7a8651d</t>
+          <t>id-952aef4c115d8f12</t>
         </is>
       </c>
     </row>
@@ -1474,14 +1476,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1491,22 +1493,22 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>27/2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
+          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
+          <t>16 de septiembre de 2026 - Hora: 10:00</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1520,15 +1522,19 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
+      <c r="M14" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-952aef4c115d8f12</t>
+          <t>id-608017f47f903d65</t>
         </is>
       </c>
     </row>
@@ -1543,14 +1549,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
+          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1560,22 +1566,22 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>27/2026</t>
+          <t>06/26</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
+          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>16/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>16 de septiembre de 2026 - Hora: 10:00</t>
+          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1583,7 +1589,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
+        </is>
+      </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1601,7 +1611,7 @@
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-608017f47f903d65</t>
+          <t>id-9dbdaa6090d92bd4</t>
         </is>
       </c>
     </row>
@@ -1616,14 +1626,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
+          <t>MUNICIPALIDAD DE SEGUÍ</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1633,12 +1643,12 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>06/26</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
+          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”. Apertura de Sobres 17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y entrega en Área de Suministro del Municipio, y también se podrá descargar en el Sitio Oficial Digital Municipal https://www.segui.gob.ar . Edgardo Muller, Presidente Municipal. ID:52321 - F.C. 04-00075716 3 v./03/09/2026</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1648,19 +1658,15 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
+          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
-        </is>
-      </c>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1678,7 +1684,7 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-9dbdaa6090d92bd4</t>
+          <t>id-90c3d1f38f49418a</t>
         </is>
       </c>
     </row>
@@ -1693,14 +1699,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SEGUÍ</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1710,30 +1716,34 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>015/2026</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”. Apertura de Sobres 17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y entrega en Área de Suministro del Municipio, y también se podrá descargar en el Sitio Oficial Digital Municipal https://www.segui.gob.ar . Edgardo Muller, Presidente Municipal. ID:52321 - F.C. 04-00075716 3 v./03/09/2026</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y</t>
+          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
+        </is>
+      </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1751,7 +1761,7 @@
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-90c3d1f38f49418a</t>
+          <t>id-74dfdad7e5f9d048</t>
         </is>
       </c>
     </row>
@@ -1766,14 +1776,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1783,12 +1793,12 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>015/2026</t>
+          <t>09/26</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1798,7 +1808,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1808,7 +1818,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -1828,7 +1838,7 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-74dfdad7e5f9d048</t>
+          <t>id-6a4a84712fd41a03</t>
         </is>
       </c>
     </row>
@@ -1850,7 +1860,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1860,12 +1870,12 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>09/26</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
+          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1875,7 +1885,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1883,29 +1893,21 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K19" s="4" t="inlineStr"/>
       <c r="L19" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M19" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
+      <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-6a4a84712fd41a03</t>
+          <t>id-885d4847519dfd48</t>
         </is>
       </c>
     </row>
@@ -1920,14 +1922,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1935,24 +1937,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>09/2026</t>
-        </is>
-      </c>
+      <c r="F20" s="4" t="inlineStr"/>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
+          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
+          <t>24 de SEPTIEMBRE de 2026</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1960,21 +1958,29 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>Sin Cargo</t>
+        </is>
+      </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
+      <c r="M20" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-885d4847519dfd48</t>
+          <t>id-bc610b64999d147d</t>
         </is>
       </c>
     </row>
@@ -1989,14 +1995,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2004,10 +2010,14 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr"/>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>10/2026</t>
+        </is>
+      </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
+          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez realizado el depósito/transferenci</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -2017,17 +2027,17 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>24 de SEPTIEMBRE de 2026</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN N</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>Sin Cargo</t>
+          <t>Habilitación: Pesos Ochenta Mil con 0/100 - $ 80.000, 00 - Habilitació</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -2047,7 +2057,7 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-bc610b64999d147d</t>
+          <t>id-d97b43a99f1e1824</t>
         </is>
       </c>
     </row>
@@ -2069,7 +2079,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2079,12 +2089,12 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez realizado el depósito/transferenci</t>
+          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -2094,7 +2104,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN N</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2104,7 +2114,7 @@
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>Habilitación: Pesos Ochenta Mil con 0/100 - $ 80.000, 00 - Habilitació</t>
+          <t>Habilitación: Pesos Ciento Veinte Mil con 0/100 - $ 120.000, 00 - Habi</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr">
@@ -2124,7 +2134,7 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-d97b43a99f1e1824</t>
+          <t>id-f8fab7a7b3a06a2d</t>
         </is>
       </c>
     </row>
@@ -2146,7 +2156,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2156,32 +2166,32 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>Habilitación: Pesos Ciento Veinte Mil con 0/100 - $ 120.000, 00 - Habi</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
@@ -2201,7 +2211,7 @@
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-f8fab7a7b3a06a2d</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
@@ -2223,7 +2233,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2233,12 +2243,12 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -2248,7 +2258,7 @@
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2256,29 +2266,21 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K24" s="4" t="inlineStr"/>
       <c r="L24" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M24" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
+      <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
@@ -2288,9 +2290,9 @@
           <t>09/09/2026</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -2300,7 +2302,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2310,22 +2312,18 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2333,21 +2331,29 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr"/>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L25" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
+      <c r="M25" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
@@ -2362,14 +2368,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2379,18 +2385,18 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2398,11 +2404,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K26" s="4" t="inlineStr"/>
       <c r="L26" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2420,7 +2422,7 @@
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
@@ -2508,35 +2510,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Boletín Oficial</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>ENERSA convoca a la Licitación Nº 2026- 1227 con el objeto de la provi sión de postes de hormigón para líneas</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2550,15 +2552,19 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr"/>
+      <c r="M28" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-e90021854bcee649</t>
         </is>
       </c>
     </row>
@@ -2590,18 +2596,18 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2623,7 +2629,7 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
@@ -2655,18 +2661,18 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2688,7 +2694,7 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -2720,18 +2726,18 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2753,7 +2759,7 @@
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -2785,18 +2791,18 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2818,7 +2824,7 @@
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -2848,16 +2854,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr"/>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2879,7 +2889,7 @@
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -2909,20 +2919,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>04/2025</t>
-        </is>
-      </c>
+      <c r="F34" s="4" t="inlineStr"/>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2944,7 +2950,7 @@
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -2976,18 +2982,18 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3009,7 +3015,7 @@
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
@@ -3041,18 +3047,18 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3074,7 +3080,7 @@
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
@@ -3111,13 +3117,13 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3139,7 +3145,7 @@
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
@@ -3161,28 +3167,28 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3199,12 +3205,12 @@
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
@@ -3219,29 +3225,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>499/26</t>
+          <t>01/26</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA Nº 499/26: EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
@@ -3264,12 +3270,12 @@
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-f53eab44dba8d43f</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
@@ -3284,9 +3290,9 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C40" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -3296,17 +3302,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>235/26</t>
+          <t>499/26</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>Licitación Privada N° 235/26: reparación de cenefas en losas pórticos</t>
+          <t>LICITACIÓN PÚBLICA Nº 499/26: EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
@@ -3334,7 +3340,7 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-22f9c51cdaebefb7</t>
+          <t>id-f53eab44dba8d43f</t>
         </is>
       </c>
     </row>
@@ -3361,17 +3367,17 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación Privada</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>498/26</t>
+          <t>235/26</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA N° 498/26: reparación de un tramo del cerramiento perimetral del Túnel Subfluvial</t>
+          <t>Licitación Privada N° 235/26: reparación de cenefas en losas pórticos</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
@@ -3399,7 +3405,7 @@
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-46d81e3efd2ae483</t>
+          <t>id-22f9c51cdaebefb7</t>
         </is>
       </c>
     </row>
@@ -3421,7 +3427,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Túnel Subfluvial</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3431,18 +3437,18 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>10-2026</t>
+          <t>498/26</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+          <t>LICITACIÓN PÚBLICA N° 498/26: reparación de un tramo del cerramiento perimetral del Túnel Subfluvial</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
@@ -3459,12 +3465,12 @@
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Túnel Subfluvial</t>
         </is>
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
-          <t>id-bdd0abb0374c3f42</t>
+          <t>id-46d81e3efd2ae483</t>
         </is>
       </c>
     </row>
@@ -3479,35 +3485,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C43" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>09-2026</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
@@ -3524,12 +3530,12 @@
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
-          <t>id-42c411be9946d956</t>
+          <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
@@ -3556,17 +3562,17 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>10-2026</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr"/>
@@ -3594,12 +3600,142 @@
       </c>
       <c r="O44" s="4" t="inlineStr">
         <is>
+          <t>id-bdd0abb0374c3f42</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>09-2026</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr"/>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego — figura como Pendiente</t>
+        </is>
+      </c>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K45" s="4" t="inlineStr"/>
+      <c r="L45" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="O45" s="4" t="inlineStr">
+        <is>
+          <t>id-42c411be9946d956</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Licitación Privada</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>04-2026</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr"/>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego — figura como Pendiente</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K46" s="4" t="inlineStr"/>
+      <c r="L46" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="O46" s="4" t="inlineStr">
+        <is>
           <t>id-023b6b75e7014a9c</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O44"/>
+  <autoFilter ref="A1:O46"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3624,8 +3760,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId28"/>
@@ -3635,8 +3771,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId39"/>
@@ -3644,29 +3780,32 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId69"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Reconocer los tipos de llamado abreviados en el Boletín
Santa Elena publicó 'Lic. Pca. N° 08/2026' (un camión con caja volcadora por
$129M) y el parser descartaba el bloque entero por no encontrar la palabra
'licitación' completa. En ese mismo boletín 15 avisos la escriben completa y
sólo ese la abrevia.

Ahora se aceptan Lic. Pca. / Lic. Púb. / Lic. Priv. y se muestran con el nombre
completo. También se lee 'VALOR DE PLIEGOS' en plural y el objeto ya no arrastra
el '-PRESUPUESTO:' pegado con guión.

Recupera además el camión usado de la Comuna de La Picada y el vehículo 0 km de
Herrera. Vigentes: 23 -> 25.
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$48</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O46"/>
+  <dimension ref="A1:O48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1922,14 +1922,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1937,20 +1937,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr"/>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>07/2026</t>
+        </is>
+      </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
+          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>24 de SEPTIEMBRE de 2026</t>
+          <t>21/09/2026 HORA: 10:00 HS</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1960,7 +1964,7 @@
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>Sin Cargo</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -1980,7 +1984,7 @@
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-bc610b64999d147d</t>
+          <t>id-6ddfa0f2f1aa296d</t>
         </is>
       </c>
     </row>
@@ -1995,14 +1999,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2010,14 +2014,10 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>10/2026</t>
-        </is>
-      </c>
+      <c r="F21" s="4" t="inlineStr"/>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez realizado el depósito/transferenci</t>
+          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -2027,17 +2027,17 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN N</t>
+          <t>24 de SEPTIEMBRE de 2026</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>Habilitación: Pesos Ochenta Mil con 0/100 - $ 80.000, 00 - Habilitació</t>
+          <t>Sin Cargo</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -2057,7 +2057,7 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-d97b43a99f1e1824</t>
+          <t>id-bc610b64999d147d</t>
         </is>
       </c>
     </row>
@@ -2079,7 +2079,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2089,12 +2089,12 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez</t>
+          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez realizado el depósito/transferenci</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -2104,7 +2104,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN N</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2112,11 +2112,7 @@
           <t>17/09/2026</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>Habilitación: Pesos Ciento Veinte Mil con 0/100 - $ 120.000, 00 - Habi</t>
-        </is>
-      </c>
+      <c r="K22" s="4" t="inlineStr"/>
       <c r="L22" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2134,7 +2130,7 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-f8fab7a7b3a06a2d</t>
+          <t>id-d97b43a99f1e1824</t>
         </is>
       </c>
     </row>
@@ -2156,7 +2152,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2166,34 +2162,30 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr"/>
       <c r="L23" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2211,7 +2203,7 @@
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-f8fab7a7b3a06a2d</t>
         </is>
       </c>
     </row>
@@ -2226,14 +2218,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2243,22 +2235,22 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
+          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCLUIDO</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2266,21 +2258,29 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr"/>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L24" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
+      <c r="M24" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-1590925c21c7e363</t>
         </is>
       </c>
     </row>
@@ -2290,9 +2290,9 @@
           <t>09/09/2026</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -2302,7 +2302,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2312,18 +2312,22 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr"/>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2333,7 +2337,7 @@
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr">
@@ -2353,7 +2357,7 @@
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
@@ -2363,19 +2367,19 @@
           <t>09/09/2026</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C26" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2385,18 +2389,22 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr"/>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2410,19 +2418,15 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M26" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
+      <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
@@ -2437,14 +2441,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2454,18 +2458,18 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2475,7 +2479,7 @@
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>s in cargo Consultas: comprascomuna6to@hotmail.com Celular: 3444- 4493</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr">
@@ -2495,7 +2499,7 @@
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-511256e6329e386a</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
@@ -2517,22 +2521,22 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Boletín Oficial</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>ENERSA convoca a la Licitación Nº 2026- 1227 con el objeto de la provi sión de postes de hormigón para líneas</t>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
@@ -2564,7 +2568,7 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-e90021854bcee649</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
@@ -2579,14 +2583,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2596,18 +2600,18 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2621,15 +2625,19 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr"/>
+      <c r="M29" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
@@ -2644,35 +2652,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Boletín Oficial</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>ENERSA convoca a la Licitación Nº 2026- 1227 con el objeto de la provi sión de postes de hormigón para líneas</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2686,15 +2694,19 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr"/>
+      <c r="M30" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-e90021854bcee649</t>
         </is>
       </c>
     </row>
@@ -2726,18 +2738,18 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2759,7 +2771,7 @@
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
@@ -2791,18 +2803,18 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2824,7 +2836,7 @@
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -2856,18 +2868,18 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2889,7 +2901,7 @@
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -2919,16 +2931,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr"/>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2950,7 +2966,7 @@
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -2982,18 +2998,18 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>04/2025</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3015,7 +3031,7 @@
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -3045,20 +3061,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>03/2025</t>
-        </is>
-      </c>
+      <c r="F36" s="4" t="inlineStr"/>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3080,7 +3092,7 @@
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -3112,18 +3124,18 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3145,7 +3157,7 @@
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
@@ -3177,18 +3189,18 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3210,7 +3222,7 @@
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
@@ -3232,28 +3244,28 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3270,12 +3282,12 @@
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
@@ -3290,14 +3302,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C40" s="7" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3307,18 +3319,18 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>499/26</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA Nº 499/26: EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
@@ -3335,12 +3347,12 @@
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-f53eab44dba8d43f</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
@@ -3355,29 +3367,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C41" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>235/26</t>
+          <t>01/26</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>Licitación Privada N° 235/26: reparación de cenefas en losas pórticos</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
@@ -3400,12 +3412,12 @@
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-22f9c51cdaebefb7</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
@@ -3420,9 +3432,9 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C42" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -3437,12 +3449,12 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>498/26</t>
+          <t>499/26</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA N° 498/26: reparación de un tramo del cerramiento perimetral del Túnel Subfluvial</t>
+          <t>LICITACIÓN PÚBLICA Nº 499/26: EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
@@ -3470,7 +3482,7 @@
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
-          <t>id-46d81e3efd2ae483</t>
+          <t>id-f53eab44dba8d43f</t>
         </is>
       </c>
     </row>
@@ -3485,29 +3497,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C43" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>Túnel Subfluvial</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Privada</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>235/26</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>Licitación Privada N° 235/26: reparación de cenefas en losas pórticos</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
@@ -3530,12 +3542,12 @@
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>Túnel Subfluvial</t>
         </is>
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
-          <t>id-0691eb485d7548eb</t>
+          <t>id-22f9c51cdaebefb7</t>
         </is>
       </c>
     </row>
@@ -3557,7 +3569,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Túnel Subfluvial</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -3567,18 +3579,18 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>10-2026</t>
+          <t>498/26</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+          <t>LICITACIÓN PÚBLICA N° 498/26: reparación de un tramo del cerramiento perimetral del Túnel Subfluvial</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr"/>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
@@ -3595,12 +3607,12 @@
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Túnel Subfluvial</t>
         </is>
       </c>
       <c r="O44" s="4" t="inlineStr">
         <is>
-          <t>id-bdd0abb0374c3f42</t>
+          <t>id-46d81e3efd2ae483</t>
         </is>
       </c>
     </row>
@@ -3615,35 +3627,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C45" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>09-2026</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr"/>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr">
@@ -3660,12 +3672,12 @@
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
-          <t>id-42c411be9946d956</t>
+          <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
@@ -3692,17 +3704,17 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>10-2026</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr"/>
@@ -3730,12 +3742,142 @@
       </c>
       <c r="O46" s="4" t="inlineStr">
         <is>
+          <t>id-bdd0abb0374c3f42</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>09-2026</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr"/>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego — figura como Pendiente</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K47" s="4" t="inlineStr"/>
+      <c r="L47" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="O47" s="4" t="inlineStr">
+        <is>
+          <t>id-42c411be9946d956</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Licitación Privada</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>04-2026</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="inlineStr"/>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego — figura como Pendiente</t>
+        </is>
+      </c>
+      <c r="J48" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K48" s="4" t="inlineStr"/>
+      <c r="L48" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="O48" s="4" t="inlineStr">
+        <is>
           <t>id-023b6b75e7014a9c</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O46"/>
+  <autoFilter ref="A1:O48"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3780,32 +3922,36 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId73"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Objeto recortado y enlace directo al pliego del organismo
Dos mejoras sobre los avisos del Boletín:

- El objeto se llevaba el aviso entero hasta el ID porque el corte sólo
  reconocía rótulos EN MAYÚSCULAS con dos puntos, y muchos siguen con
  'Apertura de Sobres 17/09/2026' o 'El pliego será gratuito'.
- El aviso menciona la web del organismo pero no el enlace al PDF del pliego.
  Ahora, para las vigentes sin pliego propio, se entra a esa web y se busca el
  PDF por el número de licitación (08/2026 aparece como 08-2026, 8-2026...).
  Con pliego propio del organismo: 2 -> 24. Si no aparece, queda el boletín.
- 'El pliego será Gratuito' también cuenta como valor del pliego.
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -1453,7 +1453,11 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
+      <c r="M13" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N13" t="inlineStr">
         <is>
           <t>Min. Planeamiento (provincia)</t>
@@ -1648,7 +1652,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”. Apertura de Sobres 17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y entrega en Área de Suministro del Municipio, y también se podrá descargar en el Sitio Oficial Digital Municipal https://www.segui.gob.ar . Edgardo Muller, Presidente Municipal. ID:52321 - F.C. 04-00075716 3 v./03/09/2026</t>
+          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1658,12 +1662,12 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal. El pliego será Gratuito. El mismo se encontrará para su consulta y</t>
+          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr"/>
@@ -1899,7 +1903,11 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr"/>
+      <c r="M19" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N19" t="inlineStr">
         <is>
           <t>Min. Planeamiento (provincia)</t>
@@ -2094,7 +2102,7 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez realizado el depósito/transferenci</t>
+          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -2104,7 +2112,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN N</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2167,7 +2175,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G. Apertura de Ofertas: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.- Venta de Pliegos - Habilitación a la Licitación: Desde el 03 de septiembre del año 2026 y hasta el día 17 de septiembre del año 2026, inclusive. Una vez</t>
+          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -2177,7 +2185,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2418,7 +2426,11 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
+      <c r="M26" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N26" t="inlineStr">
         <is>
           <t>Min. Planeamiento (provincia)</t>
@@ -2763,7 +2775,11 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr"/>
+      <c r="M31" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N31" t="inlineStr">
         <is>
           <t>IAPV — Viviendas</t>
@@ -2828,7 +2844,11 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr"/>
+      <c r="M32" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N32" t="inlineStr">
         <is>
           <t>IAPV — Viviendas</t>
@@ -2893,7 +2913,11 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr"/>
+      <c r="M33" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N33" t="inlineStr">
         <is>
           <t>IAPV — Viviendas</t>
@@ -2958,7 +2982,11 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr"/>
+      <c r="M34" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N34" t="inlineStr">
         <is>
           <t>IAPV — Viviendas</t>
@@ -3023,7 +3051,11 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr"/>
+      <c r="M35" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N35" t="inlineStr">
         <is>
           <t>IAPV — Viviendas</t>
@@ -3084,7 +3116,11 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr"/>
+      <c r="M36" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N36" t="inlineStr">
         <is>
           <t>IAPV — Viviendas</t>
@@ -3149,7 +3185,11 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr"/>
+      <c r="M37" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N37" t="inlineStr">
         <is>
           <t>IAPV — Viviendas</t>
@@ -3214,7 +3254,11 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr"/>
+      <c r="M38" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N38" t="inlineStr">
         <is>
           <t>IAPV — Viviendas</t>
@@ -3279,7 +3323,11 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr"/>
+      <c r="M39" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N39" t="inlineStr">
         <is>
           <t>IAPV — Viviendas</t>
@@ -3344,7 +3392,11 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr"/>
+      <c r="M40" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N40" t="inlineStr">
         <is>
           <t>IAPV — Viviendas</t>
@@ -3409,7 +3461,11 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr"/>
+      <c r="M41" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N41" t="inlineStr">
         <is>
           <t>Vialidad Entre Ríos (DPV)</t>
@@ -3474,7 +3530,11 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr"/>
+      <c r="M42" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N42" t="inlineStr">
         <is>
           <t>Túnel Subfluvial</t>
@@ -3539,7 +3599,11 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr"/>
+      <c r="M43" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N43" t="inlineStr">
         <is>
           <t>Túnel Subfluvial</t>
@@ -3604,7 +3668,11 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr"/>
+      <c r="M44" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N44" t="inlineStr">
         <is>
           <t>Túnel Subfluvial</t>
@@ -3669,7 +3737,11 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr"/>
+      <c r="M45" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N45" t="inlineStr">
         <is>
           <t>ENERSA</t>
@@ -3734,7 +3806,11 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr"/>
+      <c r="M46" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N46" t="inlineStr">
         <is>
           <t>CAFESG (Salto Grande)</t>
@@ -3799,7 +3875,11 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr"/>
+      <c r="M47" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N47" t="inlineStr">
         <is>
           <t>CAFESG (Salto Grande)</t>
@@ -3864,7 +3944,11 @@
           <t>ver licitación</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr"/>
+      <c r="M48" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
       <c r="N48" t="inlineStr">
         <is>
           <t>CAFESG (Salto Grande)</t>
@@ -3902,56 +3986,77 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId94"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Reconocer 'Gratuito' con mayúscula inicial en el valor del pliego
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -1670,7 +1670,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>Gratuito</t>
+        </is>
+      </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>

</xml_diff>

<commit_message>
Leer la fecha de apertura del Túnel y el pliego del IAPV
- El Túnel escribe 'Apertura / Fecha: 14/07/26' y el patrón exigía dos puntos
  justo después de APERTURA. Ahora tolera texto en el medio y se lee el
  contenido completo del post, no sólo el resumen. Cuatro licitaciones del
  Túnel pasaron de 'revisar fecha' a tener fecha real.
- El IAPV publica los datos en una IMAGEN: la página no tiene ni fecha ni
  presupuesto. Ahora se entra al artículo para traer el PDF del pliego (las 10
  lo tienen) y se prepara la lectura de la foto con OCR.
- El workflow instala tesseract. Si no está disponible, se avisa una sola vez y
  el resto sigue funcionando.
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O48"/>
+  <dimension ref="A1:O46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -880,14 +880,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NOGOYA — COMUNA DISTRITO SAUCE -- NOGOYA</t>
+          <t>Túnel Subfluvial</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -897,22 +897,22 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>1/26</t>
+          <t>499/26</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Convocar para la adquisi ción de un Tractor agrícola 0 km, con las siguientes características técnicas: potencia de motor de 130 a 150 HP; doble Tracción, 6 (seis) cilindros; y demás especificación que se encuentran en el pliego de Especificaciones Técnicas</t>
+          <t>LICITACIÓN PÚBLICA Nº 499/26: EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Viernes 11 de Septiembre de 2026- a las 10:00 horas en la Sede Comunal de Comuna Distrito Sauce</t>
+          <t>10/09/26</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -920,11 +920,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sin costo. Solicitar en la Sede Comunal de Distrito Sauce Nogoya o al </t>
-        </is>
-      </c>
+      <c r="K6" s="4" t="inlineStr"/>
       <c r="L6" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -937,12 +933,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Túnel Subfluvial</t>
         </is>
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-328f5a2f67c14702</t>
+          <t>id-f53eab44dba8d43f</t>
         </is>
       </c>
     </row>
@@ -964,22 +960,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>NOGOYA — COMUNA DISTRITO SAUCE -- NOGOYA</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>77/2026</t>
+          <t>1/26</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICION DE CAMIONETAS</t>
+          <t>Convocar para la adquisi ción de un Tractor agrícola 0 km, con las siguientes características técnicas: potencia de motor de 130 a 150 HP; doble Tracción, 6 (seis) cilindros; y demás especificación que se encuentran en el pliego de Especificaciones Técnicas</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -989,7 +985,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>11-09-2026 08:00</t>
+          <t>Viernes 11 de Septiembre de 2026- a las 10:00 horas en la Sede Comunal de Comuna Distrito Sauce</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -997,7 +993,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr"/>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sin costo. Solicitar en la Sede Comunal de Distrito Sauce Nogoya o al </t>
+        </is>
+      </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1010,12 +1010,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-dff70529581309e6</t>
+          <t>id-328f5a2f67c14702</t>
         </is>
       </c>
     </row>
@@ -1030,39 +1030,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>06/2026</t>
+          <t>77/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Transporte de dos mil metros cúbicos (2.000 m³) de ripio arcilloso destinados al mantenimiento y mejoramiento de caminos de la jurisdicción comunal de acuerdo a los Pliegos de Bases, C ondiciones Particulares y demás documentación</t>
+          <t>ADQUISICION DE CAMIONETAS</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>14 de septiembre de 2026 - Hora: 10:00</t>
+          <t>11-09-2026 08:00</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1083,12 +1083,12 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-85e6cfd11c8a8889</t>
+          <t>id-dff70529581309e6</t>
         </is>
       </c>
     </row>
@@ -1103,29 +1103,29 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>76/2026</t>
+          <t>06/2026</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>ADQUICION DE CAMIONES COMPACTADORES DE CARGA TRASERA RSU</t>
+          <t>Transporte de dos mil metros cúbicos (2.000 m³) de ripio arcilloso destinados al mantenimiento y mejoramiento de caminos de la jurisdicción comunal de acuerdo a los Pliegos de Bases, C ondiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>14-09-2026 08:00</t>
+          <t>14 de septiembre de 2026 - Hora: 10:00</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-ccdfae2a7ede4696</t>
+          <t>id-85e6cfd11c8a8889</t>
         </is>
       </c>
     </row>
@@ -1183,32 +1183,32 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE HERRERA — DPTO. URUGUAY, ENTRE RÍOS</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>76/2026</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de vehículo 0 km destinado al traslado de personas tipo van, con capacidad para 11 plazas (1 conductor + 10 pasajeros), motorización a nafta/diesel, según pliego de espec ificaciones técnicas</t>
+          <t>ADQUICION DE CAMIONES COMPACTADORES DE CARGA TRASERA RSU</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 15/09/2026, a las 11:00 hs. en el Edificio Municipal de Herrera, sito en Av. H. Bozzolo, Nº 165,</t>
+          <t>14-09-2026 08:00</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1216,11 +1216,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K10" s="4" t="inlineStr"/>
       <c r="L10" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1233,12 +1229,12 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-28313c7a9524d0ee</t>
+          <t>id-ccdfae2a7ede4696</t>
         </is>
       </c>
     </row>
@@ -1253,14 +1249,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
+          <t>MUNICIPALIDAD DE HERRERA — DPTO. URUGUAY, ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1270,12 +1266,12 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>014/2026</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
+          <t>Adquisición de vehículo 0 km destinado al traslado de personas tipo van, con capacidad para 11 plazas (1 conductor + 10 pasajeros), motorización a nafta/diesel, según pliego de espec ificaciones técnicas</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1285,7 +1281,7 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>DE LAS OFERTAS: el día 15/09/2026, a las 11:00 hs. en el Edificio Municipal de Herrera, sito en Av. H. Bozzolo, Nº 165,</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1295,7 +1291,7 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -1315,7 +1311,7 @@
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-9e58cc9ec0b69356</t>
+          <t>id-28313c7a9524d0ee</t>
         </is>
       </c>
     </row>
@@ -1330,14 +1326,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO E INFRAESTRUCTURA</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1347,12 +1343,12 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>014/2026</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “NUEVA INSTALACION ELECTRICA, CUBIERTA DE TECHO Y REFACCION DE BAÑOS ESCUELA Nº 1 “JOSE MARIA TEXIER” -SAN SALVADOR-DEPARTAMENTO SAN SALVADOR.”</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1362,7 +1358,7 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 15 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1372,7 +1368,7 @@
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -1392,7 +1388,7 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-fb80c8ade7a8651d</t>
+          <t>id-9e58cc9ec0b69356</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1410,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>MINISTERIO DE PLANEAMIENTO E INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1424,12 +1420,12 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “NUEVA INSTALACION ELECTRICA, CUBIERTA DE TECHO Y REFACCION DE BAÑOS ESCUELA Nº 1 “JOSE MARIA TEXIER” -SAN SALVADOR-DEPARTAMENTO SAN SALVADOR.”</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1439,7 +1435,7 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
+          <t>DE LAS OFERTAS: el día 15 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1447,7 +1443,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr"/>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1460,12 +1460,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-952aef4c115d8f12</t>
+          <t>id-fb80c8ade7a8651d</t>
         </is>
       </c>
     </row>
@@ -1480,14 +1480,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1497,22 +1497,22 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>27/2026</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
+          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>16/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>16 de septiembre de 2026 - Hora: 10:00</t>
+          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1533,12 +1533,12 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-608017f47f903d65</t>
+          <t>id-952aef4c115d8f12</t>
         </is>
       </c>
     </row>
@@ -1553,14 +1553,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
+          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1570,22 +1570,22 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>06/26</t>
+          <t>27/2026</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
+          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
+          <t>16 de septiembre de 2026 - Hora: 10:00</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1593,11 +1593,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
-        </is>
-      </c>
+      <c r="K15" s="4" t="inlineStr"/>
       <c r="L15" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1615,7 +1611,7 @@
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-9dbdaa6090d92bd4</t>
+          <t>id-608017f47f903d65</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1633,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SEGUÍ</t>
+          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1647,12 +1643,12 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>06/26</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”</t>
+          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1662,7 +1658,7 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal</t>
+          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1672,7 +1668,7 @@
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>Gratuito</t>
+          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">
@@ -1692,7 +1688,7 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-90c3d1f38f49418a</t>
+          <t>id-9dbdaa6090d92bd4</t>
         </is>
       </c>
     </row>
@@ -1707,14 +1703,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
+          <t>MUNICIPALIDAD DE SEGUÍ</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1724,22 +1720,22 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>015/2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
+          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1749,7 +1745,7 @@
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
+          <t>Gratuito</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr">
@@ -1769,7 +1765,7 @@
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-74dfdad7e5f9d048</t>
+          <t>id-90c3d1f38f49418a</t>
         </is>
       </c>
     </row>
@@ -1784,14 +1780,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1801,12 +1797,12 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>09/26</t>
+          <t>015/2026</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1816,7 +1812,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1826,7 +1822,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -1846,7 +1842,7 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-6a4a84712fd41a03</t>
+          <t>id-74dfdad7e5f9d048</t>
         </is>
       </c>
     </row>
@@ -1868,7 +1864,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1878,12 +1874,12 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>09/26</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1893,7 +1889,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
+          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1901,7 +1897,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr"/>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L19" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1914,12 +1914,12 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-885d4847519dfd48</t>
+          <t>id-6a4a84712fd41a03</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1951,22 +1951,22 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
+          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026 HORA: 10:00 HS</t>
+          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1974,11 +1974,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K20" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K20" s="4" t="inlineStr"/>
       <c r="L20" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1991,12 +1987,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-6ddfa0f2f1aa296d</t>
+          <t>id-885d4847519dfd48</t>
         </is>
       </c>
     </row>
@@ -2011,14 +2007,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2026,20 +2022,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr"/>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>07/2026</t>
+        </is>
+      </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
+          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>24 de SEPTIEMBRE de 2026</t>
+          <t>21/09/2026 HORA: 10:00 HS</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2049,7 +2049,7 @@
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>Sin Cargo</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-bc610b64999d147d</t>
+          <t>id-6ddfa0f2f1aa296d</t>
         </is>
       </c>
     </row>
@@ -2084,14 +2084,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2099,14 +2099,10 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>10/2026</t>
-        </is>
-      </c>
+      <c r="F22" s="4" t="inlineStr"/>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -2116,15 +2112,19 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
+          <t>24 de SEPTIEMBRE de 2026</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="K22" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>Sin Cargo</t>
+        </is>
+      </c>
       <c r="L22" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2142,7 +2142,7 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-d97b43a99f1e1824</t>
+          <t>id-bc610b64999d147d</t>
         </is>
       </c>
     </row>
@@ -2164,7 +2164,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2174,12 +2174,12 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2215,7 +2215,7 @@
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-f8fab7a7b3a06a2d</t>
+          <t>id-d97b43a99f1e1824</t>
         </is>
       </c>
     </row>
@@ -2230,14 +2230,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2247,34 +2247,30 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCLUIDO</t>
+          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr"/>
       <c r="L24" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2292,7 +2288,7 @@
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-1590925c21c7e363</t>
+          <t>id-f8fab7a7b3a06a2d</t>
         </is>
       </c>
     </row>
@@ -2307,14 +2303,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2324,22 +2320,22 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCLUIDO</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2349,7 +2345,7 @@
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr">
@@ -2369,7 +2365,7 @@
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-1590925c21c7e363</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2387,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2401,12 +2397,12 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -2416,7 +2412,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2424,7 +2420,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr"/>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L26" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2437,12 +2437,12 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
@@ -2452,9 +2452,9 @@
           <t>09/09/2026</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2474,18 +2474,22 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr"/>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2493,11 +2497,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K27" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K27" s="4" t="inlineStr"/>
       <c r="L27" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2510,12 +2510,12 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
@@ -2530,14 +2530,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C28" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2547,18 +2547,18 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2566,7 +2566,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr"/>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L28" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2584,7 +2588,7 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
@@ -2599,14 +2603,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2616,12 +2620,12 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
@@ -2653,7 +2657,7 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-511256e6329e386a</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
@@ -2668,29 +2672,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Boletín Oficial</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>ENERSA convoca a la Licitación Nº 2026- 1227 con el objeto de la provi sión de postes de hormigón para líneas</t>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
@@ -2722,7 +2726,7 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-e90021854bcee649</t>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
@@ -2737,35 +2741,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Boletín Oficial</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>ENERSA convoca a la Licitación Nº 2026- 1227 con el objeto de la provi sión de postes de hormigón para líneas</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2786,12 +2790,12 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-e90021854bcee649</t>
         </is>
       </c>
     </row>
@@ -2823,18 +2827,18 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2860,7 +2864,7 @@
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
@@ -2892,18 +2896,18 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2929,7 +2933,7 @@
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -2961,18 +2965,18 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2998,7 +3002,7 @@
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -3030,18 +3034,18 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3067,7 +3071,7 @@
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -3097,16 +3101,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr"/>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3132,7 +3140,7 @@
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -3162,20 +3170,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>04/2025</t>
-        </is>
-      </c>
+      <c r="F37" s="4" t="inlineStr"/>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3201,7 +3205,7 @@
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -3233,18 +3237,18 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3270,7 +3274,7 @@
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
@@ -3302,18 +3306,18 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3339,7 +3343,7 @@
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
@@ -3376,13 +3380,13 @@
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
@@ -3408,7 +3412,7 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
@@ -3430,28 +3434,28 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -3472,12 +3476,12 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
@@ -3492,29 +3496,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C42" s="7" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>499/26</t>
+          <t>01/26</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA Nº 499/26: EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
@@ -3541,12 +3545,12 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
-          <t>id-f53eab44dba8d43f</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
@@ -3561,29 +3565,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C43" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>235/26</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>Licitación Privada N° 235/26: reparación de cenefas en losas pórticos</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
@@ -3610,12 +3614,12 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
-          <t>id-22f9c51cdaebefb7</t>
+          <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
@@ -3637,7 +3641,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -3647,18 +3651,18 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>498/26</t>
+          <t>10-2026</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA N° 498/26: reparación de un tramo del cerramiento perimetral del Túnel Subfluvial</t>
+          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr"/>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Ver pliego — figura como Pendiente</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
@@ -3679,12 +3683,12 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O44" s="4" t="inlineStr">
         <is>
-          <t>id-46d81e3efd2ae483</t>
+          <t>id-bdd0abb0374c3f42</t>
         </is>
       </c>
     </row>
@@ -3699,35 +3703,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C45" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>09-2026</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr"/>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Ver pliego — figura como Pendiente</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr">
@@ -3748,12 +3752,12 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
-          <t>id-0691eb485d7548eb</t>
+          <t>id-42c411be9946d956</t>
         </is>
       </c>
     </row>
@@ -3780,17 +3784,17 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación Privada</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>10-2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr"/>
@@ -3822,150 +3826,12 @@
       </c>
       <c r="O46" s="4" t="inlineStr">
         <is>
-          <t>id-bdd0abb0374c3f42</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>09/09/2026</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C47" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>CAFESG (Salto Grande)</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>09-2026</t>
-        </is>
-      </c>
-      <c r="G47" s="5" t="inlineStr">
-        <is>
-          <t>REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
-        </is>
-      </c>
-      <c r="H47" s="4" t="inlineStr"/>
-      <c r="I47" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego — figura como Pendiente</t>
-        </is>
-      </c>
-      <c r="J47" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K47" s="4" t="inlineStr"/>
-      <c r="L47" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M47" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>CAFESG (Salto Grande)</t>
-        </is>
-      </c>
-      <c r="O47" s="4" t="inlineStr">
-        <is>
-          <t>id-42c411be9946d956</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>09/09/2026</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C48" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>CAFESG (Salto Grande)</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Licitación Privada</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>04-2026</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr">
-        <is>
-          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
-        </is>
-      </c>
-      <c r="H48" s="4" t="inlineStr"/>
-      <c r="I48" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego — figura como Pendiente</t>
-        </is>
-      </c>
-      <c r="J48" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K48" s="4" t="inlineStr"/>
-      <c r="L48" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M48" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>CAFESG (Salto Grande)</t>
-        </is>
-      </c>
-      <c r="O48" s="4" t="inlineStr">
-        <is>
           <t>id-023b6b75e7014a9c</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O48"/>
+  <autoFilter ref="A1:O46"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -4057,10 +3923,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId88"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId89"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId94"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 10/09/2026 08:00
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O38"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -657,14 +657,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>FEDERACION — COMUNA DE SAN PEDRO -- DEPARTAMENTO DE FEDERACIÓN</t>
+          <t>CONCORDIA — MUNICIPALIDAD DE PUERTO YERUA</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -674,22 +674,22 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>1/2026</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>“PROVISION RIPIO SELECCIONADO EN ORIGEN Y ENTREGADO SOBRE TRANSPORTE”</t>
+          <t>Adquisición de una motoniveladora 0 Km</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>09 de Septiembre de 2026 - 10:00 hs</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -697,11 +697,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>Sin costo</t>
-        </is>
-      </c>
+      <c r="K3" s="4" t="inlineStr"/>
       <c r="L3" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -719,7 +715,7 @@
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>id-719cc55444d8579b</t>
+          <t>id-61b6e4f9568150b0</t>
         </is>
       </c>
     </row>
@@ -734,14 +730,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>CONCORDIA — MUNICIPALIDAD DE PUERTO YERUA</t>
+          <t>ENTE INTERPROVINCIAL TUNEL SUBFLUVIAL RAUL URANGA -- CARLOS S. BEGNIS</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -749,14 +745,10 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>1/2026</t>
-        </is>
-      </c>
+      <c r="F4" s="4" t="inlineStr"/>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de una motoniveladora 0 Km</t>
+          <t>EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -774,7 +766,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>GRATUITO FECHA DE APERTURA: 10/09/2026</t>
+        </is>
+      </c>
       <c r="L4" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -792,7 +788,7 @@
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>id-61b6e4f9568150b0</t>
+          <t>id-439ddd7aaa7f7b3e</t>
         </is>
       </c>
     </row>
@@ -814,7 +810,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ENTE INTERPROVINCIAL TUNEL SUBFLUVIAL RAUL URANGA -- CARLOS S. BEGNIS</t>
+          <t>Túnel Subfluvial</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -822,10 +818,14 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr"/>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>499/26</t>
+        </is>
+      </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
+          <t>LICITACIÓN PÚBLICA Nº 499/26: EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -835,7 +835,7 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>10/09/26</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -843,11 +843,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>GRATUITO FECHA DE APERTURA: 10/09/2026</t>
-        </is>
-      </c>
+      <c r="K5" s="4" t="inlineStr"/>
       <c r="L5" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -860,12 +856,12 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Túnel Subfluvial</t>
         </is>
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-439ddd7aaa7f7b3e</t>
+          <t>id-f53eab44dba8d43f</t>
         </is>
       </c>
     </row>
@@ -880,14 +876,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>NOGOYA — COMUNA DISTRITO SAUCE -- NOGOYA</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -897,22 +893,22 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>499/26</t>
+          <t>1/26</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA Nº 499/26: EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
+          <t>Convocar para la adquisi ción de un Tractor agrícola 0 km, con las siguientes características técnicas: potencia de motor de 130 a 150 HP; doble Tracción, 6 (seis) cilindros; y demás especificación que se encuentran en el pliego de Especificaciones Técnicas</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>10/09/26</t>
+          <t>Viernes 11 de Septiembre de 2026- a las 10:00 horas en la Sede Comunal de Comuna Distrito Sauce</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -920,7 +916,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr"/>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sin costo. Solicitar en la Sede Comunal de Distrito Sauce Nogoya o al </t>
+        </is>
+      </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -933,12 +933,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-f53eab44dba8d43f</t>
+          <t>id-328f5a2f67c14702</t>
         </is>
       </c>
     </row>
@@ -960,22 +960,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>NOGOYA — COMUNA DISTRITO SAUCE -- NOGOYA</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>1/26</t>
+          <t>77/2026</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Convocar para la adquisi ción de un Tractor agrícola 0 km, con las siguientes características técnicas: potencia de motor de 130 a 150 HP; doble Tracción, 6 (seis) cilindros; y demás especificación que se encuentran en el pliego de Especificaciones Técnicas</t>
+          <t>ADQUISICION DE CAMIONETAS</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -985,7 +985,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Viernes 11 de Septiembre de 2026- a las 10:00 horas en la Sede Comunal de Comuna Distrito Sauce</t>
+          <t>11-09-2026 08:00</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -993,11 +993,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sin costo. Solicitar en la Sede Comunal de Distrito Sauce Nogoya o al </t>
-        </is>
-      </c>
+      <c r="K7" s="4" t="inlineStr"/>
       <c r="L7" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1010,12 +1006,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-328f5a2f67c14702</t>
+          <t>id-dff70529581309e6</t>
         </is>
       </c>
     </row>
@@ -1030,39 +1026,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>77/2026</t>
+          <t>06/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICION DE CAMIONETAS</t>
+          <t>Transporte de dos mil metros cúbicos (2.000 m³) de ripio arcilloso destinados al mantenimiento y mejoramiento de caminos de la jurisdicción comunal de acuerdo a los Pliegos de Bases, C ondiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>11-09-2026 08:00</t>
+          <t>14 de septiembre de 2026 - Hora: 10:00</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1083,12 +1079,12 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-dff70529581309e6</t>
+          <t>id-85e6cfd11c8a8889</t>
         </is>
       </c>
     </row>
@@ -1103,29 +1099,29 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>06/2026</t>
+          <t>76/2026</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Transporte de dos mil metros cúbicos (2.000 m³) de ripio arcilloso destinados al mantenimiento y mejoramiento de caminos de la jurisdicción comunal de acuerdo a los Pliegos de Bases, C ondiciones Particulares y demás documentación</t>
+          <t>ADQUICION DE CAMIONES COMPACTADORES DE CARGA TRASERA RSU</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1135,7 +1131,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>14 de septiembre de 2026 - Hora: 10:00</t>
+          <t>14-09-2026 08:00</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1156,12 +1152,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-85e6cfd11c8a8889</t>
+          <t>id-ccdfae2a7ede4696</t>
         </is>
       </c>
     </row>
@@ -1183,32 +1179,32 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>MUNICIPALIDAD DE HERRERA — DPTO. URUGUAY, ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>76/2026</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>ADQUICION DE CAMIONES COMPACTADORES DE CARGA TRASERA RSU</t>
+          <t>Adquisición de vehículo 0 km destinado al traslado de personas tipo van, con capacidad para 11 plazas (1 conductor + 10 pasajeros), motorización a nafta/diesel, según pliego de espec ificaciones técnicas</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>14-09-2026 08:00</t>
+          <t>DE LAS OFERTAS: el día 15/09/2026, a las 11:00 hs. en el Edificio Municipal de Herrera, sito en Av. H. Bozzolo, Nº 165,</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1216,7 +1212,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1229,12 +1229,12 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-ccdfae2a7ede4696</t>
+          <t>id-28313c7a9524d0ee</t>
         </is>
       </c>
     </row>
@@ -1249,14 +1249,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE HERRERA — DPTO. URUGUAY, ENTRE RÍOS</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1266,12 +1266,12 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>014/2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de vehículo 0 km destinado al traslado de personas tipo van, con capacidad para 11 plazas (1 conductor + 10 pasajeros), motorización a nafta/diesel, según pliego de espec ificaciones técnicas</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 15/09/2026, a las 11:00 hs. en el Edificio Municipal de Herrera, sito en Av. H. Bozzolo, Nº 165,</t>
+          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -1311,7 +1311,7 @@
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-28313c7a9524d0ee</t>
+          <t>id-9e58cc9ec0b69356</t>
         </is>
       </c>
     </row>
@@ -1326,14 +1326,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
+          <t>MINISTERIO DE PLANEAMIENTO E INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1343,12 +1343,12 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>014/2026</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “NUEVA INSTALACION ELECTRICA, CUBIERTA DE TECHO Y REFACCION DE BAÑOS ESCUELA Nº 1 “JOSE MARIA TEXIER” -SAN SALVADOR-DEPARTAMENTO SAN SALVADOR.”</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1358,7 +1358,7 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>DE LAS OFERTAS: el día 15 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-9e58cc9ec0b69356</t>
+          <t>id-fb80c8ade7a8651d</t>
         </is>
       </c>
     </row>
@@ -1410,7 +1410,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO E INFRAESTRUCTURA</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1420,12 +1420,12 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “NUEVA INSTALACION ELECTRICA, CUBIERTA DE TECHO Y REFACCION DE BAÑOS ESCUELA Nº 1 “JOSE MARIA TEXIER” -SAN SALVADOR-DEPARTAMENTO SAN SALVADOR.”</t>
+          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1435,7 +1435,7 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 15 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1443,11 +1443,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K13" s="4" t="inlineStr"/>
       <c r="L13" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1460,12 +1456,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-fb80c8ade7a8651d</t>
+          <t>id-952aef4c115d8f12</t>
         </is>
       </c>
     </row>
@@ -1480,14 +1476,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1497,22 +1493,22 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>27/2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
+          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
+          <t>16 de septiembre de 2026 - Hora: 10:00</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1533,12 +1529,12 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-952aef4c115d8f12</t>
+          <t>id-608017f47f903d65</t>
         </is>
       </c>
     </row>
@@ -1553,14 +1549,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
+          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1570,22 +1566,22 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>27/2026</t>
+          <t>06/26</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
+          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>16/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>16 de septiembre de 2026 - Hora: 10:00</t>
+          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1593,7 +1589,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
+        </is>
+      </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1611,7 +1611,7 @@
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-608017f47f903d65</t>
+          <t>id-9dbdaa6090d92bd4</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
+          <t>MUNICIPALIDAD DE SEGUÍ</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1643,12 +1643,12 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>06/26</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
+          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
+          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
+          <t>Gratuito</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-9dbdaa6090d92bd4</t>
+          <t>id-90c3d1f38f49418a</t>
         </is>
       </c>
     </row>
@@ -1703,14 +1703,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SEGUÍ</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1720,22 +1720,22 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>015/2026</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal</t>
+          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>Gratuito</t>
+          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr">
@@ -1765,7 +1765,7 @@
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-90c3d1f38f49418a</t>
+          <t>id-74dfdad7e5f9d048</t>
         </is>
       </c>
     </row>
@@ -1780,14 +1780,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1797,12 +1797,12 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>015/2026</t>
+          <t>09/26</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1822,7 +1822,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-74dfdad7e5f9d048</t>
+          <t>id-6a4a84712fd41a03</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1874,12 +1874,12 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>09/26</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
+          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1897,11 +1897,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K19" s="4" t="inlineStr"/>
       <c r="L19" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1914,12 +1910,12 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-6a4a84712fd41a03</t>
+          <t>id-885d4847519dfd48</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1937,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1951,22 +1947,22 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
+          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
+          <t>21/09/2026 HORA: 10:00 HS</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1974,7 +1970,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1987,12 +1987,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-885d4847519dfd48</t>
+          <t>id-6ddfa0f2f1aa296d</t>
         </is>
       </c>
     </row>
@@ -2007,14 +2007,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2022,24 +2022,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>07/2026</t>
-        </is>
-      </c>
+      <c r="F21" s="4" t="inlineStr"/>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
+          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026 HORA: 10:00 HS</t>
+          <t>24 de SEPTIEMBRE de 2026</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2049,7 +2045,7 @@
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>Sin Cargo</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -2069,7 +2065,7 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-6ddfa0f2f1aa296d</t>
+          <t>id-bc610b64999d147d</t>
         </is>
       </c>
     </row>
@@ -2084,14 +2080,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2099,10 +2095,14 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr"/>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>10/2026</t>
+        </is>
+      </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
+          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -2112,19 +2112,15 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>24 de SEPTIEMBRE de 2026</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>Sin Cargo</t>
-        </is>
-      </c>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr"/>
       <c r="L22" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2142,7 +2138,7 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-bc610b64999d147d</t>
+          <t>id-d97b43a99f1e1824</t>
         </is>
       </c>
     </row>
@@ -2164,7 +2160,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2174,12 +2170,12 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -2189,7 +2185,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2215,7 +2211,7 @@
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-d97b43a99f1e1824</t>
+          <t>id-f8fab7a7b3a06a2d</t>
         </is>
       </c>
     </row>
@@ -2230,14 +2226,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2247,30 +2243,34 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCLUIDO</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="K24" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L24" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2288,7 +2288,7 @@
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-f8fab7a7b3a06a2d</t>
+          <t>id-1590925c21c7e363</t>
         </is>
       </c>
     </row>
@@ -2303,14 +2303,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2320,22 +2320,22 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCLUIDO</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr">
@@ -2365,7 +2365,7 @@
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-1590925c21c7e363</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2397,12 +2397,12 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2420,11 +2420,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K26" s="4" t="inlineStr"/>
       <c r="L26" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2437,12 +2433,12 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
@@ -2452,9 +2448,9 @@
           <t>09/09/2026</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
@@ -2464,7 +2460,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2474,22 +2470,18 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2497,7 +2489,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K27" s="4" t="inlineStr"/>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L27" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2510,12 +2506,12 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
@@ -2530,14 +2526,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2547,18 +2543,18 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2566,11 +2562,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K28" s="4" t="inlineStr"/>
       <c r="L28" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2588,7 +2580,7 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
@@ -2603,14 +2595,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2620,12 +2612,12 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
@@ -2657,7 +2649,7 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
@@ -2672,29 +2664,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>Boletín Oficial</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+          <t>ENERSA convoca a la Licitación Nº 2026- 1227 con el objeto de la provi sión de postes de hormigón para líneas</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
@@ -2726,14 +2718,14 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-511256e6329e386a</t>
+          <t>id-e90021854bcee649</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2741,35 +2733,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Boletín Oficial</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>ENERSA convoca a la Licitación Nº 2026- 1227 con el objeto de la provi sión de postes de hormigón para líneas</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2790,19 +2782,19 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-e90021854bcee649</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2827,18 +2819,18 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2846,11 +2838,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K32" s="4" t="inlineStr">
-        <is>
-          <t>$ 120.976,01</t>
-        </is>
-      </c>
+      <c r="K32" s="4" t="inlineStr"/>
       <c r="L32" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2868,14 +2856,14 @@
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2900,18 +2888,18 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2937,14 +2925,14 @@
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2959,28 +2947,28 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -3001,19 +2989,19 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3021,35 +3009,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C35" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3070,19 +3058,19 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-0691eb485d7548eb</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3090,14 +3078,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3105,20 +3093,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>10-2026</t>
-        </is>
-      </c>
+      <c r="F36" s="4" t="inlineStr"/>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3139,19 +3123,19 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-bdd0abb0374c3f42</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3159,14 +3143,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C37" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3176,18 +3160,18 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>09-2026</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3208,19 +3192,19 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-42c411be9946d956</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3228,35 +3212,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C38" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3277,17 +3261,500 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O38" s="4" t="inlineStr">
+        <is>
+          <t>id-75bfffae63b7eedc</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>IAPV (Vivienda)</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr"/>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>Publicada 06/10/2025 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K39" s="4" t="inlineStr"/>
+      <c r="L39" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M39" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>id-07ddb93a12c5a870</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>IAPV (Vivienda)</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>Concurso de Precio N° 02/2025</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr"/>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>Publicada 19/06/2025 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K40" s="4" t="inlineStr"/>
+      <c r="L40" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M40" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O40" s="4" t="inlineStr">
+        <is>
+          <t>id-7c1bf02160a66f67</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Concurso</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>01/26</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr"/>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K41" s="4" t="inlineStr"/>
+      <c r="L41" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M41" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="O41" s="4" t="inlineStr">
+        <is>
+          <t>id-9a16884dd5a64a49</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>ENERSA</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>2026-1227</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr"/>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr"/>
+      <c r="L42" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M42" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>ENERSA</t>
+        </is>
+      </c>
+      <c r="O42" s="4" t="inlineStr">
+        <is>
+          <t>id-0691eb485d7548eb</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
           <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
-      <c r="O38" s="4" t="inlineStr">
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>10-2026</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr"/>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego — figura como Pendiente</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr"/>
+      <c r="L43" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M43" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="O43" s="4" t="inlineStr">
+        <is>
+          <t>id-bdd0abb0374c3f42</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>09-2026</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr"/>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego — figura como Pendiente</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K44" s="4" t="inlineStr"/>
+      <c r="L44" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M44" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="O44" s="4" t="inlineStr">
+        <is>
+          <t>id-42c411be9946d956</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Licitación Privada</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>04-2026</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr"/>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego — figura como Pendiente</t>
+        </is>
+      </c>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K45" s="4" t="inlineStr"/>
+      <c r="L45" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M45" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="O45" s="4" t="inlineStr">
         <is>
           <t>id-023b6b75e7014a9c</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O38"/>
+  <autoFilter ref="A1:O45"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3363,6 +3830,20 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId88"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 11/09/2026 08:05
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O38"/>
+  <dimension ref="A1:O42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -664,7 +664,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>CONCORDIA — MUNICIPALIDAD DE PUERTO YERUA</t>
+          <t>NOGOYA — COMUNA DISTRITO SAUCE -- NOGOYA</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -674,22 +674,22 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>1/2026</t>
+          <t>1/26</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de una motoniveladora 0 Km</t>
+          <t>Convocar para la adquisi ción de un Tractor agrícola 0 km, con las siguientes características técnicas: potencia de motor de 130 a 150 HP; doble Tracción, 6 (seis) cilindros; y demás especificación que se encuentran en el pliego de Especificaciones Técnicas</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>Viernes 11 de Septiembre de 2026- a las 10:00 horas en la Sede Comunal de Comuna Distrito Sauce</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -697,7 +697,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr"/>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sin costo. Solicitar en la Sede Comunal de Distrito Sauce Nogoya o al </t>
+        </is>
+      </c>
       <c r="L3" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -715,7 +719,7 @@
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>id-61b6e4f9568150b0</t>
+          <t>id-328f5a2f67c14702</t>
         </is>
       </c>
     </row>
@@ -737,7 +741,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ENTE INTERPROVINCIAL TUNEL SUBFLUVIAL RAUL URANGA -- CARLOS S. BEGNIS</t>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -745,20 +749,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr"/>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>06/2026</t>
+        </is>
+      </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
+          <t>Transporte de dos mil metros cúbicos (2.000 m³) de ripio arcilloso destinados al mantenimiento y mejoramiento de caminos de la jurisdicción comunal de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>14 de septiembre de 2026 - Hora: 10:00</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -766,11 +774,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>GRATUITO FECHA DE APERTURA: 10/09/2026</t>
-        </is>
-      </c>
+      <c r="K4" s="4" t="inlineStr"/>
       <c r="L4" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -788,7 +792,7 @@
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>id-439ddd7aaa7f7b3e</t>
+          <t>id-85e6cfd11c8a8889</t>
         </is>
       </c>
     </row>
@@ -803,39 +807,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>499/26</t>
+          <t>76/2026</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA Nº 499/26: EXTRACCIÓN DE DEPÓSITOS DE SUELO EN SECTOR INFERIOR DEL TÚNEL SUBFLUVIAL</t>
+          <t>ADQUICION DE CAMIONES COMPACTADORES DE CARGA TRASERA RSU</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>10/09/26</t>
+          <t>14-09-2026 08:00</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -856,12 +860,12 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Túnel Subfluvial</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-f53eab44dba8d43f</t>
+          <t>id-ccdfae2a7ede4696</t>
         </is>
       </c>
     </row>
@@ -883,7 +887,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NOGOYA — COMUNA DISTRITO SAUCE -- NOGOYA</t>
+          <t>MUNICIPALIDAD DE HERRERA — DPTO. URUGUAY, ENTRE RIOS</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -893,22 +897,22 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>1/26</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Convocar para la adquisi ción de un Tractor agrícola 0 km, con las siguientes características técnicas: potencia de motor de 130 a 150 HP; doble Tracción, 6 (seis) cilindros; y demás especificación que se encuentran en el pliego de Especificaciones Técnicas</t>
+          <t>Adquisición de vehículo 0 km destinado al traslado de personas tipo van, con capacidad para 11 plazas (1 conductor + 10 pasajeros), motorización a nafta/diesel, según pliego de especificaciones técnicas</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Viernes 11 de Septiembre de 2026- a las 10:00 horas en la Sede Comunal de Comuna Distrito Sauce</t>
+          <t>DE LAS OFERTAS: el día 15/09/2026, a las 11:00 hs. en el Edificio Municipal de Herrera, sito en Av. H. Bozzolo, Nº 165,</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -918,7 +922,7 @@
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">sin costo. Solicitar en la Sede Comunal de Distrito Sauce Nogoya o al </t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
@@ -938,7 +942,7 @@
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-328f5a2f67c14702</t>
+          <t>id-28313c7a9524d0ee</t>
         </is>
       </c>
     </row>
@@ -953,39 +957,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>77/2026</t>
+          <t>014/2026</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICION DE CAMIONETAS</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>11-09-2026 08:00</t>
+          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -993,7 +997,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr"/>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
+        </is>
+      </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1006,12 +1014,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-dff70529581309e6</t>
+          <t>id-9e58cc9ec0b69356</t>
         </is>
       </c>
     </row>
@@ -1026,14 +1034,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>MINISTERIO DE PLANEAMIENTO E INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1043,22 +1051,22 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>06/2026</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Transporte de dos mil metros cúbicos (2.000 m³) de ripio arcilloso destinados al mantenimiento y mejoramiento de caminos de la jurisdicción comunal de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “NUEVA INSTALACION ELECTRICA, CUBIERTA DE TECHO Y REFACCION DE BAÑOS ESCUELA Nº 1 “JOSE MARIA TEXIER” -SAN SALVADOR-DEPARTAMENTO SAN SALVADOR.”</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>14 de septiembre de 2026 - Hora: 10:00</t>
+          <t>DE LAS OFERTAS: el día 15 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1066,7 +1074,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr"/>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1084,7 +1096,7 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-85e6cfd11c8a8889</t>
+          <t>id-fb80c8ade7a8651d</t>
         </is>
       </c>
     </row>
@@ -1099,39 +1111,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>76/2026</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>ADQUICION DE CAMIONES COMPACTADORES DE CARGA TRASERA RSU</t>
+          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>14-09-2026 08:00</t>
+          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1152,12 +1164,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-ccdfae2a7ede4696</t>
+          <t>id-952aef4c115d8f12</t>
         </is>
       </c>
     </row>
@@ -1172,14 +1184,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE HERRERA — DPTO. URUGUAY, ENTRE RIOS</t>
+          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1189,22 +1201,22 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>27/2026</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de vehículo 0 km destinado al traslado de personas tipo van, con capacidad para 11 plazas (1 conductor + 10 pasajeros), motorización a nafta/diesel, según pliego de especificaciones técnicas</t>
+          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 15/09/2026, a las 11:00 hs. en el Edificio Municipal de Herrera, sito en Av. H. Bozzolo, Nº 165,</t>
+          <t>16 de septiembre de 2026 - Hora: 10:00</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1212,11 +1224,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K10" s="4" t="inlineStr"/>
       <c r="L10" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1234,7 +1242,7 @@
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-28313c7a9524d0ee</t>
+          <t>id-608017f47f903d65</t>
         </is>
       </c>
     </row>
@@ -1249,14 +1257,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
+          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1266,22 +1274,22 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>014/2026</t>
+          <t>06/26</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
+          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1291,7 +1299,7 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
+          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -1311,7 +1319,7 @@
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-9e58cc9ec0b69356</t>
+          <t>id-9dbdaa6090d92bd4</t>
         </is>
       </c>
     </row>
@@ -1326,14 +1334,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO E INFRAESTRUCTURA</t>
+          <t>MUNICIPALIDAD DE SEGUÍ</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1343,22 +1351,22 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “NUEVA INSTALACION ELECTRICA, CUBIERTA DE TECHO Y REFACCION DE BAÑOS ESCUELA Nº 1 “JOSE MARIA TEXIER” -SAN SALVADOR-DEPARTAMENTO SAN SALVADOR.”</t>
+          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 15 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1368,7 +1376,7 @@
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>Gratuito</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -1388,7 +1396,7 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-fb80c8ade7a8651d</t>
+          <t>id-90c3d1f38f49418a</t>
         </is>
       </c>
     </row>
@@ -1403,14 +1411,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1420,22 +1428,22 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>015/2026</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
+          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1443,7 +1451,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr"/>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
+        </is>
+      </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1456,12 +1468,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-952aef4c115d8f12</t>
+          <t>id-74dfdad7e5f9d048</t>
         </is>
       </c>
     </row>
@@ -1476,14 +1488,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1493,22 +1505,22 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>27/2026</t>
+          <t>09/26</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>16/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>16 de septiembre de 2026 - Hora: 10:00</t>
+          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1516,7 +1528,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr"/>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1534,7 +1550,7 @@
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-608017f47f903d65</t>
+          <t>id-6a4a84712fd41a03</t>
         </is>
       </c>
     </row>
@@ -1549,14 +1565,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1566,22 +1582,22 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>06/26</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
+          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
+          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1589,11 +1605,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
-        </is>
-      </c>
+      <c r="K15" s="4" t="inlineStr"/>
       <c r="L15" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1606,12 +1618,12 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-9dbdaa6090d92bd4</t>
+          <t>id-885d4847519dfd48</t>
         </is>
       </c>
     </row>
@@ -1626,14 +1638,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SEGUÍ</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1643,22 +1655,22 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”</t>
+          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal</t>
+          <t>21/09/2026 HORA: 10:00 HS</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1668,7 +1680,7 @@
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>Gratuito</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">
@@ -1688,7 +1700,7 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-90c3d1f38f49418a</t>
+          <t>id-6ddfa0f2f1aa296d</t>
         </is>
       </c>
     </row>
@@ -1710,7 +1722,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1718,24 +1730,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>015/2026</t>
-        </is>
-      </c>
+      <c r="F17" s="4" t="inlineStr"/>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
+          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>24 de SEPTIEMBRE de 2026</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1745,7 +1753,7 @@
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
+          <t>Sin Cargo</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr">
@@ -1765,7 +1773,7 @@
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-74dfdad7e5f9d048</t>
+          <t>id-bc610b64999d147d</t>
         </is>
       </c>
     </row>
@@ -1787,7 +1795,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1797,34 +1805,30 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>09/26</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
+          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K18" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1842,7 +1846,7 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-6a4a84712fd41a03</t>
+          <t>id-d97b43a99f1e1824</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1868,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1879,22 +1883,22 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
+          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr"/>
@@ -1910,19 +1914,19 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-885d4847519dfd48</t>
+          <t>id-f8fab7a7b3a06a2d</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1930,49 +1934,49 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>5/2026</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
+          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026 HORA: 10:00 HS</t>
+          <t>28/9/2026 – 10:00 horas</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>$25.000,00</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -1987,12 +1991,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-6ddfa0f2f1aa296d</t>
+          <t>id-1609ce58e128c413</t>
         </is>
       </c>
     </row>
@@ -2007,14 +2011,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2022,20 +2026,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr"/>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>08/2026</t>
+        </is>
+      </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
+          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>24 de SEPTIEMBRE de 2026</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2045,7 +2053,7 @@
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>Sin Cargo</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -2065,7 +2073,7 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-bc610b64999d147d</t>
+          <t>id-1590925c21c7e363</t>
         </is>
       </c>
     </row>
@@ -2087,7 +2095,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2097,30 +2105,34 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="K22" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L22" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2138,7 +2150,7 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-d97b43a99f1e1824</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2172,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2170,27 +2182,27 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr"/>
@@ -2206,69 +2218,65 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-f8fab7a7b3a06a2d</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C24" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>5/2026</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>28/09/2026</t>
-        </is>
-      </c>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>28/9/2026 – 10:00 horas</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>$25.000,00</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L24" s="6" t="inlineStr">
@@ -2283,12 +2291,12 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-1609ce58e128c413</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
@@ -2298,19 +2306,19 @@
           <t>09/09/2026</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2320,22 +2328,18 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>29/09/2026</t>
-        </is>
-      </c>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2343,11 +2347,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K25" s="4" t="inlineStr"/>
       <c r="L25" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2365,7 +2365,7 @@
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-1590925c21c7e363</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
@@ -2375,19 +2375,19 @@
           <t>09/09/2026</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2397,22 +2397,18 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2420,11 +2416,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K26" s="4" t="inlineStr"/>
       <c r="L26" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2442,7 +2434,7 @@
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
@@ -2452,44 +2444,40 @@
           <t>09/09/2026</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>Boletín Oficial</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
+          <t>ENERSA convoca a la Licitación Nº 2026- 1227 con el objeto de la provi sión de postes de hormigón para líneas</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2510,19 +2498,19 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-e90021854bcee649</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2530,14 +2518,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2547,18 +2535,18 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2566,11 +2554,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K28" s="4" t="inlineStr"/>
       <c r="L28" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2583,19 +2567,19 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2603,14 +2587,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2620,18 +2604,18 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2652,19 +2636,19 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2672,14 +2656,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2694,13 +2678,13 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2721,19 +2705,19 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-511256e6329e386a</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2741,35 +2725,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Boletín Oficial</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>ENERSA convoca a la Licitación Nº 2026- 1227 con el objeto de la provi sión de postes de hormigón para líneas</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2790,19 +2774,19 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-e90021854bcee649</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2827,18 +2811,18 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2846,11 +2830,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K32" s="4" t="inlineStr">
-        <is>
-          <t>$ 120.976,01</t>
-        </is>
-      </c>
+      <c r="K32" s="4" t="inlineStr"/>
       <c r="L32" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2868,14 +2848,14 @@
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2898,20 +2878,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>02/2025</t>
-        </is>
-      </c>
+      <c r="F33" s="4" t="inlineStr"/>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2937,14 +2913,14 @@
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2959,28 +2935,28 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -3001,19 +2977,19 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3021,35 +2997,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C35" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3070,12 +3046,12 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-0691eb485d7548eb</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
@@ -3090,14 +3066,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3107,18 +3083,18 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>10-2026</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3139,12 +3115,12 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-bdd0abb0374c3f42</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
@@ -3159,14 +3135,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C37" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3176,18 +3152,18 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>09-2026</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3208,12 +3184,12 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-42c411be9946d956</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
@@ -3228,35 +3204,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C38" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>01/26</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3277,17 +3253,293 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="O38" s="4" t="inlineStr">
+        <is>
+          <t>id-9a16884dd5a64a49</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>ENERSA</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>2026-1227</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr"/>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K39" s="4" t="inlineStr"/>
+      <c r="L39" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M39" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>ENERSA</t>
+        </is>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>id-0691eb485d7548eb</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
           <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
-      <c r="O38" s="4" t="inlineStr">
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>10-2026</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr"/>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego — figura como Pendiente</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K40" s="4" t="inlineStr"/>
+      <c r="L40" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M40" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="O40" s="4" t="inlineStr">
+        <is>
+          <t>id-bdd0abb0374c3f42</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>09-2026</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr"/>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego — figura como Pendiente</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K41" s="4" t="inlineStr"/>
+      <c r="L41" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M41" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="O41" s="4" t="inlineStr">
+        <is>
+          <t>id-42c411be9946d956</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Licitación Privada</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>04-2026</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr"/>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego — figura como Pendiente</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr"/>
+      <c r="L42" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M42" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="O42" s="4" t="inlineStr">
         <is>
           <t>id-023b6b75e7014a9c</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O38"/>
+  <autoFilter ref="A1:O42"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3363,6 +3615,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId82"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Clasificar por lo que se contrata, unificar repetidas y estado Duplicada
- El rubro ahora sale del VERBO, no sólo de las palabras: comprar materiales
  para una obra es Materiales; ejecutar la obra es Infraestructura. Antes
  'ADQUISICIÓN DE MATERIALES PARA EL PLAN DE PAVIMENTACIÓN' caía en
  Infraestructura por la palabra pavimentación. 12/12 casos de prueba.
- Una misma licitación que llega por dos fuentes (el Boletín y la web del
  organismo) se unifica en una fila, quedándose con los datos de ambas y
  anotando las dos fuentes.
- Estado 'Duplicada' para lo que la detección automática no agarre: junto con
  'Descartada' manda la fila al fondo de la lista y la saca del Resumen.
- El Resumen muestra el seguimiento de cada próxima apertura.
- Se quitó el nombre de la empresa de todos los textos.
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:O33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -572,7 +572,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -649,7 +649,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -726,7 +726,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -872,7 +872,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE HERRERA — DPTO. URUGUAY, ENTRE RIOS</t>
+          <t>MUNICIPALIDAD DE HERRERA — DPTO. URUGUAY, ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -949,7 +949,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1103,7 +1103,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1176,7 +1176,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1249,7 +1249,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1326,7 +1326,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1403,7 +1403,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1480,7 +1480,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1557,7 +1557,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1630,7 +1630,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1707,7 +1707,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1715,9 +1715,9 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1780,7 +1780,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1853,7 +1853,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Boletín Oficial de Entre Ríos + CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
@@ -2003,7 +2003,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -2080,7 +2080,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2157,7 +2157,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2230,7 +2230,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2303,7 +2303,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2372,7 +2372,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2441,7 +2441,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2510,7 +2510,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2535,18 +2535,18 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2554,7 +2554,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr"/>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>$ 120.976,01</t>
+        </is>
+      </c>
       <c r="L28" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2572,14 +2576,14 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2604,18 +2608,18 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2641,14 +2645,14 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2663,28 +2667,28 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>01/26</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2705,19 +2709,19 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2725,35 +2729,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2774,19 +2778,19 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2794,14 +2798,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2811,18 +2815,18 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>10-2026</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Ver pliego — figura como Pendiente</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2843,19 +2847,19 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-bdd0abb0374c3f42</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2863,31 +2867,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr"/>
+          <t>Licitación Privada</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>04-2026</t>
+        </is>
+      </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Ver pliego — figura como Pendiente</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2908,638 +2916,17 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>10/09/2026</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>IAPV (Vivienda)</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>04/2025</t>
-        </is>
-      </c>
-      <c r="G34" s="5" t="inlineStr">
-        <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
-        </is>
-      </c>
-      <c r="H34" s="4" t="inlineStr"/>
-      <c r="I34" s="4" t="inlineStr">
-        <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
-        </is>
-      </c>
-      <c r="J34" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K34" s="4" t="inlineStr"/>
-      <c r="L34" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M34" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>IAPV — Viviendas</t>
-        </is>
-      </c>
-      <c r="O34" s="4" t="inlineStr">
-        <is>
-          <t>id-34c85bcdb9b1123f</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>10/09/2026</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>IAPV (Vivienda)</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>03/2025</t>
-        </is>
-      </c>
-      <c r="G35" s="5" t="inlineStr">
-        <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
-        </is>
-      </c>
-      <c r="H35" s="4" t="inlineStr"/>
-      <c r="I35" s="4" t="inlineStr">
-        <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
-        </is>
-      </c>
-      <c r="J35" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K35" s="4" t="inlineStr"/>
-      <c r="L35" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M35" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>IAPV — Viviendas</t>
-        </is>
-      </c>
-      <c r="O35" s="4" t="inlineStr">
-        <is>
-          <t>id-75bfffae63b7eedc</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>09/09/2026</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>IAPV (Vivienda)</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>02/2025</t>
-        </is>
-      </c>
-      <c r="G36" s="5" t="inlineStr">
-        <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
-        </is>
-      </c>
-      <c r="H36" s="4" t="inlineStr"/>
-      <c r="I36" s="4" t="inlineStr">
-        <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
-        </is>
-      </c>
-      <c r="J36" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K36" s="4" t="inlineStr"/>
-      <c r="L36" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M36" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t>IAPV — Viviendas</t>
-        </is>
-      </c>
-      <c r="O36" s="4" t="inlineStr">
-        <is>
-          <t>id-07ddb93a12c5a870</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>09/09/2026</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>IAPV (Vivienda)</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>02/2025</t>
-        </is>
-      </c>
-      <c r="G37" s="5" t="inlineStr">
-        <is>
-          <t>Concurso de Precio N° 02/2025</t>
-        </is>
-      </c>
-      <c r="H37" s="4" t="inlineStr"/>
-      <c r="I37" s="4" t="inlineStr">
-        <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
-        </is>
-      </c>
-      <c r="J37" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K37" s="4" t="inlineStr"/>
-      <c r="L37" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M37" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>IAPV — Viviendas</t>
-        </is>
-      </c>
-      <c r="O37" s="4" t="inlineStr">
-        <is>
-          <t>id-7c1bf02160a66f67</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>09/09/2026</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Concurso</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>01/26</t>
-        </is>
-      </c>
-      <c r="G38" s="5" t="inlineStr">
-        <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
-        </is>
-      </c>
-      <c r="H38" s="4" t="inlineStr"/>
-      <c r="I38" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J38" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K38" s="4" t="inlineStr"/>
-      <c r="L38" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M38" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="O38" s="4" t="inlineStr">
-        <is>
-          <t>id-9a16884dd5a64a49</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>09/09/2026</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C39" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>ENERSA</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>2026-1227</t>
-        </is>
-      </c>
-      <c r="G39" s="5" t="inlineStr">
-        <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
-        </is>
-      </c>
-      <c r="H39" s="4" t="inlineStr"/>
-      <c r="I39" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J39" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K39" s="4" t="inlineStr"/>
-      <c r="L39" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M39" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>ENERSA</t>
-        </is>
-      </c>
-      <c r="O39" s="4" t="inlineStr">
-        <is>
-          <t>id-0691eb485d7548eb</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>09/09/2026</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C40" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>CAFESG (Salto Grande)</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="inlineStr">
-        <is>
-          <t>10-2026</t>
-        </is>
-      </c>
-      <c r="G40" s="5" t="inlineStr">
-        <is>
-          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
-        </is>
-      </c>
-      <c r="H40" s="4" t="inlineStr"/>
-      <c r="I40" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego — figura como Pendiente</t>
-        </is>
-      </c>
-      <c r="J40" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K40" s="4" t="inlineStr"/>
-      <c r="L40" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M40" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>CAFESG (Salto Grande)</t>
-        </is>
-      </c>
-      <c r="O40" s="4" t="inlineStr">
-        <is>
-          <t>id-bdd0abb0374c3f42</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>09/09/2026</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C41" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>CAFESG (Salto Grande)</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>09-2026</t>
-        </is>
-      </c>
-      <c r="G41" s="5" t="inlineStr">
-        <is>
-          <t>REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
-        </is>
-      </c>
-      <c r="H41" s="4" t="inlineStr"/>
-      <c r="I41" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego — figura como Pendiente</t>
-        </is>
-      </c>
-      <c r="J41" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K41" s="4" t="inlineStr"/>
-      <c r="L41" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M41" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>CAFESG (Salto Grande)</t>
-        </is>
-      </c>
-      <c r="O41" s="4" t="inlineStr">
-        <is>
-          <t>id-42c411be9946d956</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>09/09/2026</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C42" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>CAFESG (Salto Grande)</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Licitación Privada</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>04-2026</t>
-        </is>
-      </c>
-      <c r="G42" s="5" t="inlineStr">
-        <is>
-          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
-        </is>
-      </c>
-      <c r="H42" s="4" t="inlineStr"/>
-      <c r="I42" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego — figura como Pendiente</t>
-        </is>
-      </c>
-      <c r="J42" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K42" s="4" t="inlineStr"/>
-      <c r="L42" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M42" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>CAFESG (Salto Grande)</t>
-        </is>
-      </c>
-      <c r="O42" s="4" t="inlineStr">
-        <is>
           <t>id-023b6b75e7014a9c</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O42"/>
+  <autoFilter ref="A1:O33"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3605,24 +2992,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId82"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>